<commit_message>
Updated excel - Water
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Preneeth O\Desktop\shwetashubham\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D36D386-84B3-4371-90A5-61C442590945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D994AB9C-F136-4FF9-A6F4-6B967CA5F7E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="9" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="READ ME FIRST" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1169" uniqueCount="697">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1173" uniqueCount="700">
   <si>
     <t>HOW TO USE THIS SHEET</t>
   </si>
@@ -1671,15 +1671,6 @@
     <t>extended</t>
   </si>
   <si>
-    <t>Ravinder B</t>
-  </si>
-  <si>
-    <t>E-302</t>
-  </si>
-  <si>
-    <t>91777 62227</t>
-  </si>
-  <si>
     <t>Gajendra B</t>
   </si>
   <si>
@@ -2146,6 +2137,24 @@
   </si>
   <si>
     <t>Check what support staff cover, then raise a Ticket in NoBrokerHood App.</t>
+  </si>
+  <si>
+    <t>Sarvesh Kumar Collure</t>
+  </si>
+  <si>
+    <t>90009 99086</t>
+  </si>
+  <si>
+    <t>F- 503</t>
+  </si>
+  <si>
+    <t>AGBM/2026/SEP</t>
+  </si>
+  <si>
+    <t>The Water Fund shall be utilized for procuring water through tankers and for other water replenishment initiatives and projects.</t>
+  </si>
+  <si>
+    <t>Water Fund Utilization</t>
   </si>
 </sst>
 </file>
@@ -2181,8 +2190,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2523,78 +2533,78 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B64"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="78.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -2602,7 +2612,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -2610,7 +2620,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -2618,17 +2628,17 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -2636,7 +2646,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -2644,7 +2654,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -2652,7 +2662,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>24</v>
       </c>
@@ -2660,7 +2670,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>26</v>
       </c>
@@ -2668,7 +2678,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>28</v>
       </c>
@@ -2676,7 +2686,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>30</v>
       </c>
@@ -2684,7 +2694,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>32</v>
       </c>
@@ -2692,7 +2702,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>34</v>
       </c>
@@ -2700,7 +2710,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>36</v>
       </c>
@@ -2708,7 +2718,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>38</v>
       </c>
@@ -2716,7 +2726,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>40</v>
       </c>
@@ -2724,7 +2734,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>42</v>
       </c>
@@ -2732,7 +2742,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>44</v>
       </c>
@@ -2740,7 +2750,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>46</v>
       </c>
@@ -2748,17 +2758,17 @@
         <v>47</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>49</v>
       </c>
@@ -2766,7 +2776,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>51</v>
       </c>
@@ -2774,7 +2784,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>53</v>
       </c>
@@ -2782,22 +2792,22 @@
         <v>54</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>57</v>
       </c>
@@ -2805,7 +2815,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>49</v>
       </c>
@@ -2813,7 +2823,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>53</v>
       </c>
@@ -2821,37 +2831,37 @@
         <v>59</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>65</v>
       </c>
@@ -2859,7 +2869,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>67</v>
       </c>
@@ -2867,7 +2877,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>69</v>
       </c>
@@ -2875,7 +2885,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="54" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>71</v>
       </c>
@@ -2883,7 +2893,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="55" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>73</v>
       </c>
@@ -2891,7 +2901,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>75</v>
       </c>
@@ -2899,42 +2909,42 @@
         <v>76</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="59" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="61" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="62" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="63" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>81</v>
       </c>
@@ -2950,7 +2960,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -2980,7 +2990,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>478</v>
       </c>
@@ -3000,7 +3010,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>478</v>
       </c>
@@ -3020,7 +3030,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>478</v>
       </c>
@@ -3040,7 +3050,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>478</v>
       </c>
@@ -3060,7 +3070,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>478</v>
       </c>
@@ -3080,7 +3090,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>478</v>
       </c>
@@ -3100,7 +3110,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>478</v>
       </c>
@@ -3120,7 +3130,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>478</v>
       </c>
@@ -3140,7 +3150,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>478</v>
       </c>
@@ -3160,7 +3170,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>521</v>
       </c>
@@ -3174,7 +3184,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>521</v>
       </c>
@@ -3188,7 +3198,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>521</v>
       </c>
@@ -3202,7 +3212,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>521</v>
       </c>
@@ -3216,7 +3226,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>521</v>
       </c>
@@ -3230,95 +3240,95 @@
         <v>536</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>537</v>
       </c>
       <c r="B16" t="s">
-        <v>538</v>
+        <v>694</v>
       </c>
       <c r="D16" t="s">
-        <v>539</v>
+        <v>696</v>
       </c>
       <c r="E16" t="s">
-        <v>540</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>537</v>
       </c>
       <c r="B17" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="D17" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="E17" t="s">
-        <v>543</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>537</v>
       </c>
       <c r="B18" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="D18" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="E18" t="s">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>537</v>
       </c>
       <c r="B19" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="D19" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="E19" t="s">
-        <v>549</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>537</v>
       </c>
       <c r="B20" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="D20" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="E20" t="s">
-        <v>552</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>537</v>
       </c>
       <c r="B21" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="D21" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="E21" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F21" xr:uid="{00000000-0009-0000-0000-000009000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:F21" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:F15 A17:F21 A16 C16 F16" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3326,7 +3336,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -3335,16 +3345,16 @@
   <sheetData>
     <row r="1" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="B1" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="C1" t="s">
-        <v>558</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>93</v>
       </c>
@@ -3352,10 +3362,10 @@
         <v>95</v>
       </c>
       <c r="C2" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>99</v>
       </c>
@@ -3363,29 +3373,29 @@
         <v>101</v>
       </c>
       <c r="C3" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>558</v>
+      </c>
+      <c r="B4" t="s">
+        <v>559</v>
+      </c>
+      <c r="C4" t="s">
         <v>560</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>561</v>
-      </c>
-      <c r="B4" t="s">
-        <v>562</v>
-      </c>
-      <c r="C4" t="s">
-        <v>563</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>564</v>
       </c>
       <c r="B5" t="s">
         <v>95</v>
       </c>
       <c r="C5" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
     </row>
   </sheetData>
@@ -3400,7 +3410,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="70.83203125" customWidth="1"/>
@@ -3411,71 +3421,71 @@
         <v>108</v>
       </c>
       <c r="B1" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>564</v>
+      </c>
+      <c r="B2" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>566</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="B3" t="s">
         <v>567</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>568</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="B4" t="s">
         <v>569</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>570</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="B5" t="s">
         <v>571</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>572</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="B6" t="s">
         <v>573</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>574</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="B7" t="s">
         <v>575</v>
       </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>576</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+      <c r="B8" t="s">
         <v>577</v>
       </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>578</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+      <c r="B9" t="s">
         <v>579</v>
-      </c>
-      <c r="B8" t="s">
-        <v>580</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>581</v>
-      </c>
-      <c r="B9" t="s">
-        <v>582</v>
       </c>
     </row>
   </sheetData>
@@ -3490,7 +3500,7 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -3505,62 +3515,62 @@
         <v>69</v>
       </c>
       <c r="C1" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>581</v>
+      </c>
+      <c r="B2" t="s">
+        <v>582</v>
+      </c>
+      <c r="C2" t="s">
         <v>583</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>584</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
         <v>585</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" t="s">
         <v>586</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>587</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" t="s">
         <v>588</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>589</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="B5" t="s">
         <v>590</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C5" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>591</v>
       </c>
-      <c r="C4" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="B6" t="s">
         <v>592</v>
       </c>
-      <c r="B5" t="s">
-        <v>593</v>
-      </c>
-      <c r="C5" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>594</v>
-      </c>
-      <c r="B6" t="s">
-        <v>595</v>
-      </c>
       <c r="C6" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
     </row>
   </sheetData>
@@ -3575,7 +3585,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -3588,152 +3598,152 @@
         <v>108</v>
       </c>
       <c r="B1" t="s">
+        <v>593</v>
+      </c>
+      <c r="C1" t="s">
+        <v>594</v>
+      </c>
+      <c r="D1" t="s">
+        <v>595</v>
+      </c>
+      <c r="E1" t="s">
         <v>596</v>
       </c>
-      <c r="C1" t="s">
-        <v>597</v>
-      </c>
-      <c r="D1" t="s">
-        <v>598</v>
-      </c>
-      <c r="E1" t="s">
-        <v>599</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>312</v>
       </c>
       <c r="B2" t="s">
+        <v>597</v>
+      </c>
+      <c r="C2" t="s">
+        <v>598</v>
+      </c>
+      <c r="D2" t="s">
+        <v>599</v>
+      </c>
+      <c r="E2" t="s">
         <v>600</v>
       </c>
-      <c r="C2" t="s">
-        <v>601</v>
-      </c>
-      <c r="D2" t="s">
-        <v>602</v>
-      </c>
-      <c r="E2" t="s">
-        <v>603</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>254</v>
       </c>
       <c r="B3" t="s">
+        <v>601</v>
+      </c>
+      <c r="C3" t="s">
+        <v>602</v>
+      </c>
+      <c r="D3" t="s">
+        <v>603</v>
+      </c>
+      <c r="E3" t="s">
         <v>604</v>
       </c>
-      <c r="C3" t="s">
-        <v>605</v>
-      </c>
-      <c r="D3" t="s">
-        <v>606</v>
-      </c>
-      <c r="E3" t="s">
-        <v>607</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>250</v>
       </c>
       <c r="B4" t="s">
+        <v>605</v>
+      </c>
+      <c r="C4" t="s">
+        <v>606</v>
+      </c>
+      <c r="D4" t="s">
+        <v>607</v>
+      </c>
+      <c r="E4" t="s">
         <v>608</v>
       </c>
-      <c r="C4" t="s">
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>609</v>
       </c>
-      <c r="D4" t="s">
+      <c r="B5" t="s">
         <v>610</v>
       </c>
-      <c r="E4" t="s">
+      <c r="C5" t="s">
         <v>611</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="D5" t="s">
         <v>612</v>
       </c>
-      <c r="B5" t="s">
+      <c r="E5" t="s">
         <v>613</v>
       </c>
-      <c r="C5" t="s">
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>614</v>
       </c>
-      <c r="D5" t="s">
+      <c r="B6" t="s">
         <v>615</v>
       </c>
-      <c r="E5" t="s">
+      <c r="C6" t="s">
         <v>616</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="D6" t="s">
         <v>617</v>
       </c>
-      <c r="B6" t="s">
+      <c r="E6" t="s">
         <v>618</v>
       </c>
-      <c r="C6" t="s">
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>619</v>
       </c>
-      <c r="D6" t="s">
+      <c r="B7" t="s">
         <v>620</v>
       </c>
-      <c r="E6" t="s">
+      <c r="C7" t="s">
         <v>621</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+      <c r="D7" t="s">
         <v>622</v>
       </c>
-      <c r="B7" t="s">
+      <c r="E7" t="s">
         <v>623</v>
       </c>
-      <c r="C7" t="s">
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>624</v>
       </c>
-      <c r="D7" t="s">
+      <c r="B8" t="s">
         <v>625</v>
       </c>
-      <c r="E7" t="s">
+      <c r="C8" t="s">
         <v>626</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+      <c r="D8" t="s">
         <v>627</v>
       </c>
-      <c r="B8" t="s">
+      <c r="E8" t="s">
         <v>628</v>
       </c>
-      <c r="C8" t="s">
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>629</v>
       </c>
-      <c r="D8" t="s">
+      <c r="B9" t="s">
         <v>630</v>
       </c>
-      <c r="E8" t="s">
+      <c r="C9" t="s">
         <v>631</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="D9" t="s">
         <v>632</v>
       </c>
-      <c r="B9" t="s">
+      <c r="E9" t="s">
         <v>633</v>
-      </c>
-      <c r="C9" t="s">
-        <v>634</v>
-      </c>
-      <c r="D9" t="s">
-        <v>635</v>
-      </c>
-      <c r="E9" t="s">
-        <v>636</v>
       </c>
     </row>
   </sheetData>
@@ -3747,8 +3757,8 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="13.83203125" customWidth="1"/>
@@ -3760,7 +3770,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="B1" t="s">
         <v>49</v>
@@ -3769,7 +3779,7 @@
         <v>108</v>
       </c>
       <c r="D1" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="E1" t="s">
         <v>51</v>
@@ -3778,147 +3788,164 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>697</v>
+      </c>
+      <c r="B2" s="1">
+        <v>46292</v>
+      </c>
+      <c r="C2" t="s">
+        <v>699</v>
+      </c>
+      <c r="D2" t="s">
+        <v>698</v>
+      </c>
+      <c r="E2" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>636</v>
+      </c>
+      <c r="B3" t="s">
+        <v>637</v>
+      </c>
+      <c r="C3" t="s">
+        <v>638</v>
+      </c>
+      <c r="D3" t="s">
         <v>639</v>
       </c>
-      <c r="B2" t="s">
+      <c r="E3" t="s">
         <v>640</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>641</v>
       </c>
-      <c r="D2" t="s">
+      <c r="B4" t="s">
         <v>642</v>
       </c>
-      <c r="E2" t="s">
+      <c r="C4" t="s">
         <v>643</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="D4" t="s">
         <v>644</v>
       </c>
-      <c r="B3" t="s">
+      <c r="E4" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>645</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B5" t="s">
         <v>646</v>
       </c>
-      <c r="D3" t="s">
+      <c r="C5" t="s">
         <v>647</v>
       </c>
-      <c r="E3" t="s">
-        <v>643</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="D5" t="s">
         <v>648</v>
       </c>
-      <c r="B4" t="s">
+      <c r="E5" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>649</v>
       </c>
-      <c r="C4" t="s">
+      <c r="B6" t="s">
         <v>650</v>
       </c>
-      <c r="D4" t="s">
+      <c r="C6" t="s">
         <v>651</v>
       </c>
-      <c r="E4" t="s">
-        <v>643</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="D6" t="s">
         <v>652</v>
       </c>
-      <c r="B5" t="s">
+      <c r="E6" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>653</v>
       </c>
-      <c r="C5" t="s">
+      <c r="B7" t="s">
         <v>654</v>
       </c>
-      <c r="D5" t="s">
+      <c r="C7" t="s">
         <v>655</v>
       </c>
-      <c r="E5" t="s">
-        <v>643</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="D7" t="s">
         <v>656</v>
       </c>
-      <c r="B6" t="s">
+      <c r="E7" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>657</v>
       </c>
-      <c r="C6" t="s">
+      <c r="B8" t="s">
         <v>658</v>
       </c>
-      <c r="D6" t="s">
+      <c r="C8" t="s">
         <v>659</v>
       </c>
-      <c r="E6" t="s">
-        <v>643</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+      <c r="D8" t="s">
         <v>660</v>
       </c>
-      <c r="B7" t="s">
+      <c r="E8" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>661</v>
       </c>
-      <c r="C7" t="s">
+      <c r="B9" t="s">
         <v>662</v>
       </c>
-      <c r="D7" t="s">
+      <c r="C9" t="s">
         <v>663</v>
       </c>
-      <c r="E7" t="s">
-        <v>643</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+      <c r="D9" t="s">
         <v>664</v>
       </c>
-      <c r="B8" t="s">
+      <c r="E9" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>665</v>
       </c>
-      <c r="C8" t="s">
+      <c r="B10" t="s">
         <v>666</v>
       </c>
-      <c r="D8" t="s">
+      <c r="C10" t="s">
         <v>667</v>
       </c>
-      <c r="E8" t="s">
-        <v>643</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="D10" t="s">
         <v>668</v>
       </c>
-      <c r="B9" t="s">
+      <c r="E10" t="s">
         <v>669</v>
       </c>
-      <c r="C9" t="s">
-        <v>670</v>
-      </c>
-      <c r="D9" t="s">
-        <v>671</v>
-      </c>
-      <c r="E9" t="s">
-        <v>672</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F9" xr:uid="{00000000-0009-0000-0000-00000E000000}"/>
+  <autoFilter ref="A1:F10" xr:uid="{00000000-0009-0000-0000-00000E000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:F9" numberStoredAsText="1"/>
+    <ignoredError sqref="A3:F10 A1:F1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3926,7 +3953,7 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.83203125" customWidth="1"/>
     <col min="2" max="2" width="13.83203125" customWidth="1"/>
@@ -3952,29 +3979,29 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>670</v>
+      </c>
+      <c r="B2" t="s">
+        <v>637</v>
+      </c>
+      <c r="C2" t="s">
+        <v>671</v>
+      </c>
+      <c r="D2" t="s">
+        <v>672</v>
+      </c>
+      <c r="E2" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>673</v>
       </c>
-      <c r="B2" t="s">
-        <v>640</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B3" t="s">
         <v>674</v>
-      </c>
-      <c r="D2" t="s">
-        <v>675</v>
-      </c>
-      <c r="E2" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>676</v>
-      </c>
-      <c r="B3" t="s">
-        <v>677</v>
       </c>
       <c r="C3" t="s">
         <v>116</v>
@@ -3983,109 +4010,109 @@
         <v>117</v>
       </c>
       <c r="E3" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>675</v>
+      </c>
+      <c r="B4" t="s">
+        <v>676</v>
+      </c>
+      <c r="C4" t="s">
+        <v>677</v>
+      </c>
+      <c r="D4" t="s">
         <v>678</v>
       </c>
-      <c r="B4" t="s">
+      <c r="E4" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>670</v>
+      </c>
+      <c r="B5" t="s">
         <v>679</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C5" t="s">
         <v>680</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D5" t="s">
         <v>681</v>
       </c>
-      <c r="E4" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="E5" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>673</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
         <v>682</v>
-      </c>
-      <c r="C5" t="s">
-        <v>683</v>
-      </c>
-      <c r="D5" t="s">
-        <v>684</v>
-      </c>
-      <c r="E5" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>676</v>
-      </c>
-      <c r="B6" t="s">
-        <v>685</v>
       </c>
       <c r="C6" t="s">
         <v>120</v>
       </c>
       <c r="D6" t="s">
+        <v>683</v>
+      </c>
+      <c r="E6" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>670</v>
+      </c>
+      <c r="B7" t="s">
+        <v>684</v>
+      </c>
+      <c r="C7" t="s">
+        <v>685</v>
+      </c>
+      <c r="D7" t="s">
         <v>686</v>
       </c>
-      <c r="E6" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+      <c r="E7" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>675</v>
+      </c>
+      <c r="B8" t="s">
+        <v>687</v>
+      </c>
+      <c r="C8" t="s">
+        <v>688</v>
+      </c>
+      <c r="D8" t="s">
+        <v>689</v>
+      </c>
+      <c r="E8" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>673</v>
       </c>
-      <c r="B7" t="s">
-        <v>687</v>
-      </c>
-      <c r="C7" t="s">
-        <v>688</v>
-      </c>
-      <c r="D7" t="s">
-        <v>689</v>
-      </c>
-      <c r="E7" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>678</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="B9" t="s">
         <v>690</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C9" t="s">
         <v>691</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D9" t="s">
         <v>692</v>
       </c>
-      <c r="E8" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>676</v>
-      </c>
-      <c r="B9" t="s">
-        <v>693</v>
-      </c>
-      <c r="C9" t="s">
-        <v>694</v>
-      </c>
-      <c r="D9" t="s">
-        <v>695</v>
-      </c>
       <c r="E9" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
     </row>
   </sheetData>
@@ -4100,7 +4127,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="70.83203125" customWidth="1"/>
@@ -4114,7 +4141,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>84</v>
       </c>
@@ -4122,7 +4149,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>86</v>
       </c>
@@ -4130,7 +4157,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>88</v>
       </c>
@@ -4138,7 +4165,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>90</v>
       </c>
@@ -4146,7 +4173,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>92</v>
       </c>
@@ -4154,7 +4181,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>94</v>
       </c>
@@ -4162,7 +4189,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -4170,7 +4197,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>98</v>
       </c>
@@ -4178,7 +4205,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>100</v>
       </c>
@@ -4186,7 +4213,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>102</v>
       </c>
@@ -4194,7 +4221,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>104</v>
       </c>
@@ -4214,7 +4241,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -4236,7 +4263,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>110</v>
       </c>
@@ -4250,7 +4277,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>114</v>
       </c>
@@ -4264,7 +4291,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>118</v>
       </c>
@@ -4290,7 +4317,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:A15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
   </cols>
@@ -4300,72 +4327,72 @@
         <v>122</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>136</v>
       </c>
@@ -4382,7 +4409,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -4404,7 +4431,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>138</v>
       </c>
@@ -4418,7 +4445,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>142</v>
       </c>
@@ -4432,7 +4459,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>146</v>
       </c>
@@ -4446,7 +4473,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>150</v>
       </c>
@@ -4454,13 +4481,13 @@
         <v>151</v>
       </c>
       <c r="C5" t="s">
-        <v>696</v>
+        <v>693</v>
       </c>
       <c r="D5" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>153</v>
       </c>
@@ -4474,7 +4501,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>157</v>
       </c>
@@ -4488,7 +4515,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>161</v>
       </c>
@@ -4502,7 +4529,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>165</v>
       </c>
@@ -4516,7 +4543,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>169</v>
       </c>
@@ -4530,7 +4557,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>173</v>
       </c>
@@ -4556,7 +4583,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -4574,7 +4601,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>179</v>
       </c>
@@ -4585,7 +4612,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>181</v>
       </c>
@@ -4596,7 +4623,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>184</v>
       </c>
@@ -4607,7 +4634,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>187</v>
       </c>
@@ -4618,7 +4645,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>190</v>
       </c>
@@ -4629,7 +4656,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>193</v>
       </c>
@@ -4640,7 +4667,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>196</v>
       </c>
@@ -4651,7 +4678,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>198</v>
       </c>
@@ -4662,7 +4689,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>201</v>
       </c>
@@ -4673,7 +4700,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>204</v>
       </c>
@@ -4696,7 +4723,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:F139"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -4725,7 +4752,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>212</v>
       </c>
@@ -4742,7 +4769,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>212</v>
       </c>
@@ -4753,7 +4780,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>212</v>
       </c>
@@ -4764,7 +4791,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>212</v>
       </c>
@@ -4775,7 +4802,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>212</v>
       </c>
@@ -4786,7 +4813,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>212</v>
       </c>
@@ -4797,7 +4824,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>212</v>
       </c>
@@ -4808,7 +4835,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>212</v>
       </c>
@@ -4819,7 +4846,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>212</v>
       </c>
@@ -4830,7 +4857,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>224</v>
       </c>
@@ -4847,7 +4874,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>224</v>
       </c>
@@ -4858,7 +4885,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>224</v>
       </c>
@@ -4869,7 +4896,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>224</v>
       </c>
@@ -4880,7 +4907,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>224</v>
       </c>
@@ -4891,7 +4918,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>224</v>
       </c>
@@ -4902,7 +4929,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>233</v>
       </c>
@@ -4919,7 +4946,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>233</v>
       </c>
@@ -4930,7 +4957,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>233</v>
       </c>
@@ -4941,7 +4968,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>233</v>
       </c>
@@ -4952,7 +4979,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>240</v>
       </c>
@@ -4969,7 +4996,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>240</v>
       </c>
@@ -4980,7 +5007,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>240</v>
       </c>
@@ -4991,7 +5018,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>240</v>
       </c>
@@ -5002,7 +5029,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>240</v>
       </c>
@@ -5013,7 +5040,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>240</v>
       </c>
@@ -5024,7 +5051,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>240</v>
       </c>
@@ -5035,7 +5062,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>240</v>
       </c>
@@ -5046,7 +5073,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>240</v>
       </c>
@@ -5057,7 +5084,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>240</v>
       </c>
@@ -5068,7 +5095,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>240</v>
       </c>
@@ -5079,7 +5106,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>240</v>
       </c>
@@ -5090,7 +5117,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>240</v>
       </c>
@@ -5101,7 +5128,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>240</v>
       </c>
@@ -5112,7 +5139,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>240</v>
       </c>
@@ -5123,7 +5150,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>240</v>
       </c>
@@ -5134,7 +5161,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>240</v>
       </c>
@@ -5145,7 +5172,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>240</v>
       </c>
@@ -5156,7 +5183,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>240</v>
       </c>
@@ -5167,7 +5194,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>240</v>
       </c>
@@ -5178,7 +5205,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>240</v>
       </c>
@@ -5189,7 +5216,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>240</v>
       </c>
@@ -5200,7 +5227,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>240</v>
       </c>
@@ -5211,7 +5238,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>240</v>
       </c>
@@ -5222,7 +5249,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>240</v>
       </c>
@@ -5233,7 +5260,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>240</v>
       </c>
@@ -5244,7 +5271,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>240</v>
       </c>
@@ -5255,7 +5282,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>240</v>
       </c>
@@ -5266,7 +5293,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="49" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>240</v>
       </c>
@@ -5277,7 +5304,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="50" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>240</v>
       </c>
@@ -5288,7 +5315,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>273</v>
       </c>
@@ -5305,7 +5332,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="52" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>273</v>
       </c>
@@ -5316,7 +5343,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="53" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>273</v>
       </c>
@@ -5327,7 +5354,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="54" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>273</v>
       </c>
@@ -5338,7 +5365,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="55" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>273</v>
       </c>
@@ -5349,7 +5376,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="56" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>273</v>
       </c>
@@ -5360,7 +5387,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="57" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>273</v>
       </c>
@@ -5371,7 +5398,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="58" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>273</v>
       </c>
@@ -5382,7 +5409,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="59" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>273</v>
       </c>
@@ -5393,7 +5420,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="60" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>273</v>
       </c>
@@ -5404,7 +5431,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="61" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>273</v>
       </c>
@@ -5415,7 +5442,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="62" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>273</v>
       </c>
@@ -5426,7 +5453,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="63" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>273</v>
       </c>
@@ -5437,7 +5464,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="64" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>273</v>
       </c>
@@ -5448,7 +5475,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="65" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>273</v>
       </c>
@@ -5459,7 +5486,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="66" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>273</v>
       </c>
@@ -5470,7 +5497,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="67" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>273</v>
       </c>
@@ -5481,7 +5508,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="68" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>273</v>
       </c>
@@ -5492,7 +5519,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="69" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>273</v>
       </c>
@@ -5503,7 +5530,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="70" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>273</v>
       </c>
@@ -5514,7 +5541,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="71" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>273</v>
       </c>
@@ -5525,7 +5552,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="72" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>273</v>
       </c>
@@ -5536,7 +5563,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="73" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>273</v>
       </c>
@@ -5547,7 +5574,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="74" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>273</v>
       </c>
@@ -5558,7 +5585,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="75" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>273</v>
       </c>
@@ -5569,7 +5596,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="76" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>273</v>
       </c>
@@ -5580,7 +5607,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="77" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>273</v>
       </c>
@@ -5591,7 +5618,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="78" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>273</v>
       </c>
@@ -5602,7 +5629,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="79" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>273</v>
       </c>
@@ -5613,7 +5640,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="80" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>273</v>
       </c>
@@ -5624,7 +5651,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="81" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>273</v>
       </c>
@@ -5635,7 +5662,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="82" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>273</v>
       </c>
@@ -5646,7 +5673,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="83" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>308</v>
       </c>
@@ -5666,7 +5693,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="84" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>308</v>
       </c>
@@ -5677,7 +5704,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="85" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>308</v>
       </c>
@@ -5688,7 +5715,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="86" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>308</v>
       </c>
@@ -5699,7 +5726,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="87" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>308</v>
       </c>
@@ -5710,7 +5737,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="88" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>308</v>
       </c>
@@ -5721,7 +5748,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="89" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>308</v>
       </c>
@@ -5732,7 +5759,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="90" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>308</v>
       </c>
@@ -5743,7 +5770,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="91" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>308</v>
       </c>
@@ -5754,7 +5781,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="92" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>308</v>
       </c>
@@ -5765,7 +5792,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="93" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>308</v>
       </c>
@@ -5776,7 +5803,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="94" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>323</v>
       </c>
@@ -5793,7 +5820,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="95" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>323</v>
       </c>
@@ -5804,7 +5831,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="96" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>323</v>
       </c>
@@ -5815,7 +5842,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="97" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>323</v>
       </c>
@@ -5826,7 +5853,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="98" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>323</v>
       </c>
@@ -5837,7 +5864,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="99" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>323</v>
       </c>
@@ -5848,7 +5875,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="100" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>323</v>
       </c>
@@ -5859,7 +5886,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="101" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>323</v>
       </c>
@@ -5870,7 +5897,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="102" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>323</v>
       </c>
@@ -5881,7 +5908,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="103" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>323</v>
       </c>
@@ -5892,7 +5919,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="104" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>323</v>
       </c>
@@ -5903,7 +5930,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="105" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>323</v>
       </c>
@@ -5914,7 +5941,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="106" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>323</v>
       </c>
@@ -5925,7 +5952,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="107" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>323</v>
       </c>
@@ -5936,7 +5963,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="108" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>323</v>
       </c>
@@ -5947,7 +5974,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="109" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>323</v>
       </c>
@@ -5958,7 +5985,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="110" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>323</v>
       </c>
@@ -5969,7 +5996,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="111" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>323</v>
       </c>
@@ -5980,7 +6007,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="112" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>323</v>
       </c>
@@ -5991,7 +6018,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="113" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>323</v>
       </c>
@@ -6002,7 +6029,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="114" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>346</v>
       </c>
@@ -6019,7 +6046,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="115" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>346</v>
       </c>
@@ -6030,7 +6057,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="116" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>346</v>
       </c>
@@ -6041,7 +6068,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="117" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>346</v>
       </c>
@@ -6052,7 +6079,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="118" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>346</v>
       </c>
@@ -6063,7 +6090,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="119" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>346</v>
       </c>
@@ -6074,7 +6101,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="120" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>355</v>
       </c>
@@ -6091,7 +6118,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="121" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>355</v>
       </c>
@@ -6102,7 +6129,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="122" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>355</v>
       </c>
@@ -6113,7 +6140,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="123" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>355</v>
       </c>
@@ -6124,7 +6151,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="124" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>362</v>
       </c>
@@ -6141,7 +6168,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="125" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>362</v>
       </c>
@@ -6152,7 +6179,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="126" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>362</v>
       </c>
@@ -6163,7 +6190,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="127" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>362</v>
       </c>
@@ -6174,7 +6201,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="128" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>362</v>
       </c>
@@ -6185,7 +6212,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="129" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>362</v>
       </c>
@@ -6196,7 +6223,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="130" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>371</v>
       </c>
@@ -6213,7 +6240,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="131" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>371</v>
       </c>
@@ -6224,7 +6251,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="132" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>371</v>
       </c>
@@ -6235,7 +6262,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="133" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>371</v>
       </c>
@@ -6246,7 +6273,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="134" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>371</v>
       </c>
@@ -6257,7 +6284,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="135" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>371</v>
       </c>
@@ -6268,7 +6295,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="136" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>380</v>
       </c>
@@ -6285,7 +6312,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="137" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>380</v>
       </c>
@@ -6296,7 +6323,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="138" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>380</v>
       </c>
@@ -6307,7 +6334,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="139" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>380</v>
       </c>
@@ -6330,7 +6357,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:D37"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -6352,7 +6379,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>389</v>
       </c>
@@ -6366,7 +6393,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>389</v>
       </c>
@@ -6380,7 +6407,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>389</v>
       </c>
@@ -6394,7 +6421,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>389</v>
       </c>
@@ -6408,7 +6435,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>389</v>
       </c>
@@ -6422,7 +6449,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>389</v>
       </c>
@@ -6436,7 +6463,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>389</v>
       </c>
@@ -6450,7 +6477,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>400</v>
       </c>
@@ -6464,7 +6491,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>400</v>
       </c>
@@ -6478,7 +6505,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>400</v>
       </c>
@@ -6492,7 +6519,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>400</v>
       </c>
@@ -6506,7 +6533,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>400</v>
       </c>
@@ -6520,7 +6547,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>400</v>
       </c>
@@ -6534,7 +6561,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>400</v>
       </c>
@@ -6548,7 +6575,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>409</v>
       </c>
@@ -6562,7 +6589,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>409</v>
       </c>
@@ -6576,7 +6603,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>409</v>
       </c>
@@ -6590,7 +6617,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>409</v>
       </c>
@@ -6604,7 +6631,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>409</v>
       </c>
@@ -6618,7 +6645,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>409</v>
       </c>
@@ -6632,7 +6659,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>417</v>
       </c>
@@ -6646,7 +6673,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>417</v>
       </c>
@@ -6660,7 +6687,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>417</v>
       </c>
@@ -6674,7 +6701,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>417</v>
       </c>
@@ -6688,7 +6715,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>417</v>
       </c>
@@ -6702,7 +6729,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>417</v>
       </c>
@@ -6716,7 +6743,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>425</v>
       </c>
@@ -6730,7 +6757,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>425</v>
       </c>
@@ -6744,7 +6771,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>425</v>
       </c>
@@ -6758,7 +6785,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>425</v>
       </c>
@@ -6772,7 +6799,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>425</v>
       </c>
@@ -6786,7 +6813,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>425</v>
       </c>
@@ -6800,7 +6827,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>425</v>
       </c>
@@ -6814,7 +6841,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>425</v>
       </c>
@@ -6828,7 +6855,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>436</v>
       </c>
@@ -6842,7 +6869,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>436</v>
       </c>
@@ -6868,7 +6895,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -6894,7 +6921,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>443</v>
       </c>
@@ -6911,7 +6938,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>443</v>
       </c>
@@ -6928,7 +6955,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>443</v>
       </c>
@@ -6945,7 +6972,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>452</v>
       </c>
@@ -6956,7 +6983,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>452</v>
       </c>
@@ -6967,7 +6994,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>452</v>
       </c>
@@ -6978,7 +7005,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>452</v>
       </c>
@@ -6989,7 +7016,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>452</v>
       </c>
@@ -7000,7 +7027,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>452</v>
       </c>
@@ -7011,7 +7038,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>452</v>
       </c>
@@ -7022,7 +7049,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>452</v>
       </c>
@@ -7033,7 +7060,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>452</v>
       </c>
@@ -7044,7 +7071,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>452</v>
       </c>
@@ -7055,7 +7082,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>452</v>
       </c>
@@ -7066,7 +7093,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>452</v>
       </c>
@@ -7077,7 +7104,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>452</v>
       </c>

</xml_diff>

<commit_message>
Add eight guideline posters to the posters section
Adds parking, corridors, gate security, pool, gym, staff behaviour,
resident-staff interaction and save-water posters as built-in entries
alongside the existing balcony poster, and regenerates the posters
sheet tab from them.

The posters resilience tests derived their expected count from a single
hard-coded figure, so they now read the built-in count out of index.html
instead of assuming one poster.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -35,7 +35,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="11">'checklist'!A1:B9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12">'downloads'!A1:C6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13">'gallery'!A1:E9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14">'posters'!A1:C2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14">'posters'!A1:C10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15">'resolutions'!A1:F9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16">'records'!A1:E9</definedName>
   </definedNames>
@@ -1653,7 +1653,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C10"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -1682,10 +1682,98 @@
         <v>Balcony safety &amp; cleanliness — keep your balcony clean and contained, and never throw water, dust, cigarette butts or waste from balconies</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Corridors must be kept clean &amp; clear</v>
+      </c>
+      <c r="B3" t="str">
+        <v>poster-corridors.jpg</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Corridors must be kept clean &amp; clear — no footwear, cycles, furniture or storage in the common corridors. Keep the passage tidy and unobstructed for everyone.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Parking rules</v>
+      </c>
+      <c r="B4" t="str">
+        <v>poster-parking.jpg</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Park within your own allotted slot and inside the markings. No-parking zones and fire lanes are strictly enforced — vehicles are locked and fined Rs 200 a day for two-wheelers and Rs 500 for four-wheelers. No waste or storage in parking areas, and cycles belong in flat parking only.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Security at the main gate</v>
+      </c>
+      <c r="B5" t="str">
+        <v>poster-gate-security.jpg</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Residents: affix the society sticker and register your vehicle for automatic access. Guests and non-registered vehicles must use Gate 1 for entry checks. Do not misuse the entry and exit lanes — Gates 3 and 5 are planned for exit only.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Swimming pool usage rules</v>
+      </c>
+      <c r="B6" t="str">
+        <v>poster-pool.jpg</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Proper swimwear is mandatory. Children must be supervised by an adult at all times. No food or glass items near the pool. The pool is for registered residents only — guests are not allowed.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Gym guidelines</v>
+      </c>
+      <c r="B7" t="str">
+        <v>poster-gym.jpg</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Under-14s are not allowed in the gym. Do not drop weights or misuse equipment — place them gently and re-rack after use. Limit sessions to 30 minutes during peak hours so everyone gets a chance, and keep the shared audio at a moderate volume.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Residents’ behaviour towards support staff</v>
+      </c>
+      <c r="B8" t="str">
+        <v>poster-staff-behaviour.jpg</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Treat all support staff with dignity and courtesy — a smile and kind words go a long way. Do not be rude, dismissive or abusive towards support staff; mistreating them creates an unhealthy environment and is serious misconduct.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Resident &amp; support staff interaction</v>
+      </c>
+      <c r="B9" t="str">
+        <v>poster-staff-interaction.jpg</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Support staff are valued members of our society’s ecosystem and courteous interaction is expected at all times. They may not be engaged for private work inside flats beyond their defined scope. Verbal abuse, intimidation or disrespectful behaviour is strictly unacceptable — report any misconduct to the Maintenance Manager or Core Committee.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Save water — use it judiciously</v>
+      </c>
+      <c r="B10" t="str">
+        <v>poster-savewater.png</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Boond boond se banta hai kal ka savera. Close taps when not in use, use a bucket instead of a shower, run full loads in washing machines, report leaks promptly, and water plants in the morning or evening.</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C2"/>
+  <autoFilter ref="A1:C10"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C10"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
add the BGL piped-gas helpline and dial toll-free numbers correctly
The helpline renderer prefixed +91 to anything that was not a 3-5 digit
short code, so a sheet row of 1800 599 6991 dialled as a US number.
Only a bare 10-digit mobile needs the country code now; toll-free lines
and landlines are dialled exactly as written.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -27,7 +27,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2">'notices'!A1:D4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3">'festivals'!A1:A15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4">'quick_actions'!A1:D11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5">'helplines'!A1:E11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5">'helplines'!A1:E12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6">'timings'!A1:C11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7">'guidelines'!A1:F139</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8">'staff_scope'!A1:D37</definedName>
@@ -2816,7 +2816,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -2929,19 +2929,19 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Society</v>
+        <v>Emergency</v>
       </c>
       <c r="B7" t="str">
-        <v>🛠</v>
+        <v>💨</v>
       </c>
       <c r="C7" t="str">
-        <v>Maintenance Manager</v>
+        <v>Piped gas — BGL</v>
       </c>
       <c r="D7" t="str">
-        <v>97042 85706</v>
+        <v>1800 599 6991</v>
       </c>
       <c r="E7" t="str">
-        <v>All maintenance requests, 9:00 AM – 6:30 PM.</v>
+        <v>Bhagyanagar Gas, 24×7 — gas smell, leak, or any supply problem.</v>
       </c>
     </row>
     <row r="8">
@@ -2949,50 +2949,50 @@
         <v>Society</v>
       </c>
       <c r="B8" t="str">
-        <v>🛡</v>
+        <v>🛠</v>
       </c>
       <c r="C8" t="str">
-        <v>Security ASO</v>
+        <v>Maintenance Manager</v>
       </c>
       <c r="D8" t="str">
-        <v>90304 93579</v>
+        <v>97042 85706</v>
       </c>
       <c r="E8" t="str">
-        <v>Night assistance, gate issues and emergency coordination.</v>
+        <v>All maintenance requests, 9:00 AM – 6:30 PM.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Utility</v>
+        <v>Society</v>
       </c>
       <c r="B9" t="str">
-        <v>⚡</v>
+        <v>🛡</v>
       </c>
       <c r="C9" t="str">
-        <v>Electricity complaints</v>
+        <v>Security ASO</v>
       </c>
       <c r="D9" t="str">
-        <v>1912</v>
+        <v>90304 93579</v>
       </c>
       <c r="E9" t="str">
-        <v>Power failure and metering complaints (TGSPDCL).</v>
+        <v>Night assistance, gate issues and emergency coordination.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Support</v>
+        <v>Utility</v>
       </c>
       <c r="B10" t="str">
-        <v>👪</v>
+        <v>⚡</v>
       </c>
       <c r="C10" t="str">
-        <v>Childline</v>
+        <v>Electricity complaints</v>
       </c>
       <c r="D10" t="str">
-        <v>1098</v>
+        <v>1912</v>
       </c>
       <c r="E10" t="str">
-        <v>Round-the-clock help for a child in distress.</v>
+        <v>Power failure and metering complaints (TGSPDCL).</v>
       </c>
     </row>
     <row r="11">
@@ -3000,22 +3000,39 @@
         <v>Support</v>
       </c>
       <c r="B11" t="str">
+        <v>👪</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Childline</v>
+      </c>
+      <c r="D11" t="str">
+        <v>1098</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Round-the-clock help for a child in distress.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Support</v>
+      </c>
+      <c r="B12" t="str">
         <v>👩</v>
       </c>
-      <c r="C11" t="str">
+      <c r="C12" t="str">
         <v>Women’s helpline</v>
       </c>
-      <c r="D11" t="str">
+      <c r="D12" t="str">
         <v>181</v>
       </c>
-      <c r="E11" t="str">
+      <c r="E12" t="str">
         <v>Round-the-clock support and assistance for women.</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E11"/>
+  <autoFilter ref="A1:E12"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
show the festival list as a table
Fourteen name-and-date pills made for a long wrapped ribbon that
was hard to read down, and the date was easy to miss next to the
name. The same entries are now a two-column table, which lines the
dates up and matches how timings and fees are already presented.

A festival with no settled date leaves its cell empty and the
stylesheet draws a dash, so the sheet still round-trips to a blank
value rather than a literal dash the admin would have to type.

The workbook is regenerated here too, picking up the festival date
column and the BGL helpline that were waiting on a file lock.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -25,7 +25,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'settings'!A1:B13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2">'notices'!A1:D4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3">'festivals'!A1:A15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3">'festivals'!A1:B15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4">'quick_actions'!A1:D11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5">'helplines'!A1:E12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6">'timings'!A1:C11</definedName>
@@ -2554,79 +2554,119 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:B15"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="13.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
       <c r="A1" t="str">
         <v>name</v>
       </c>
+      <c r="B1" t="str">
+        <v>date</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Sankranthi</v>
+        <v>New Year</v>
+      </c>
+      <c r="B2" t="str">
+        <v>1 Jan 2027</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Republic Day</v>
+        <v>Sankranthi</v>
+      </c>
+      <c r="B3" t="str">
+        <v>15 Jan 2027</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Women's Day</v>
+        <v>Republic Day</v>
+      </c>
+      <c r="B4" t="str">
+        <v>26 Jan 2027</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Holi</v>
+        <v>Women's Day</v>
+      </c>
+      <c r="B5" t="str">
+        <v>8 Mar 2027</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Sri Rama Navami</v>
+        <v>Holi</v>
+      </c>
+      <c r="B6" t="str">
+        <v>23 Mar 2027</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
         <v>Ugadi</v>
       </c>
+      <c r="B7" t="str">
+        <v>7 Apr 2027</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Krishna Ashtami</v>
+        <v>Sri Rama Navami</v>
+      </c>
+      <c r="B8" t="str">
+        <v>15 Apr 2027</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
         <v>Independence Day</v>
       </c>
+      <c r="B9" t="str">
+        <v>15 Aug 2027</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Ganesh Chaturthi</v>
+        <v>Krishna Ashtami</v>
+      </c>
+      <c r="B10" t="str">
+        <v>25 Aug 2027</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Bathukamma</v>
+        <v>Ganesh Chaturthi</v>
+      </c>
+      <c r="B11" t="str">
+        <v>4 Sep 2027</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Ganesh Temple Anniversary</v>
+        <v>Bathukamma</v>
+      </c>
+      <c r="B12" t="str">
+        <v>30 Sep – 8 Oct 2027</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
         <v>Christmas</v>
       </c>
+      <c r="B13" t="str">
+        <v>25 Dec 2027</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>New Year</v>
+        <v>Ganesh Temple Anniversary</v>
       </c>
     </row>
     <row r="15">
@@ -2635,9 +2675,9 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A15"/>
+  <autoFilter ref="A1:B15"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
show photographs from recent society events
Adds a Latest events carousel below the committee directory, filled from a
new 'events' tab: name, date, details and a link to the picture.

The photographs live in Google Drive, whose share link opens a viewer page
rather than the image, so the file id is lifted out of whichever link shape
was pasted and rebuilt as a direct image address. Drive serves the same file
from more than one host, so the alternatives are kept and tried in turn
before the placeholder is shown.

The section and its footer link stay hidden until the tab holds a row with
both a name and a photo, so an empty carousel is never published.

Also stops a missing window.matchMedia from throwing while a carousel is
being set up, which would take down every script defined after it.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -19,8 +19,9 @@
     <sheet name="downloads" sheetId="14" r:id="rId14"/>
     <sheet name="gallery" sheetId="15" r:id="rId15"/>
     <sheet name="posters" sheetId="16" r:id="rId16"/>
-    <sheet name="resolutions" sheetId="17" r:id="rId17"/>
-    <sheet name="records" sheetId="18" r:id="rId18"/>
+    <sheet name="events" sheetId="17" r:id="rId17"/>
+    <sheet name="resolutions" sheetId="18" r:id="rId18"/>
+    <sheet name="records" sheetId="19" r:id="rId19"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'settings'!A1:B14</definedName>
@@ -38,8 +39,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="13">'downloads'!A1:C6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14">'gallery'!A1:E9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15">'posters'!A1:C10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16">'resolutions'!A1:F9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17">'records'!A1:E9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16">'events'!A1:D1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17">'resolutions'!A1:F9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18">'records'!A1:E9</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -433,7 +435,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B65"/>
+  <dimension ref="A1:B78"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="78.83203125" customWidth="1"/>
@@ -652,179 +654,179 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>resolutions</v>
+        <v>events</v>
       </c>
       <c r="B33" t="str">
-        <v>Committee / GBM decisions. Newest first is not required — the site sorts by date.</v>
+        <v>Photographs from society events. See the note below.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>records</v>
+        <v>resolutions</v>
       </c>
       <c r="B34" t="str">
-        <v>Minutes of meetings, notices and circulars. See the note below.</v>
+        <v>Committee / GBM decisions. Newest first is not required — the site sorts by date.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v/>
+        <v>records</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Minutes of meetings, notices and circulars. See the note below.</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>ABOUT THE RESOLUTIONS TAB</v>
+        <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>date</v>
-      </c>
-      <c r="B37" t="str">
-        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
+        <v>ABOUT THE EVENTS TAB</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>status</v>
+        <v>name</v>
       </c>
       <c r="B38" t="str">
-        <v>Passed / Approved / Noted / Deferred / Pending / Rejected — this sets the colour.</v>
+        <v>The event, e.g. Ganesh Chaturthi 2026. A row with no name is skipped.</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>link</v>
+        <v>date</v>
       </c>
       <c r="B39" t="str">
-        <v>Optional. A link to the full resolution PDF. Leave blank if there isn't one.</v>
+        <v>Type it as 2026-09-14 (year-month-day). The newest event is shown first.</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>The 'Latest' button shows the five most recent; 'All' shows everything.</v>
+        <v>details</v>
+      </c>
+      <c r="B40" t="str">
+        <v>A sentence or two about the day. Optional.</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v/>
+        <v>photo</v>
+      </c>
+      <c r="B41" t="str">
+        <v>The Google Drive link to the picture. A row with no photo is skipped.</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ABOUT THE RECORDS TAB</v>
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>type</v>
-      </c>
-      <c r="B43" t="str">
-        <v>mom = minutes of meeting, notice, or circular. This drives the filter buttons.</v>
+        <v>IMPORTANT: each photo in Drive must be shared as</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>date</v>
+        <v/>
       </c>
       <c r="B44" t="str">
-        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
+        <v>Share -&gt; General access -&gt; Anyone with the link -&gt; Viewer.</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>link</v>
-      </c>
-      <c r="B45" t="str">
-        <v>The PDF file name, e.g. gbm-april-2025.pdf, uploaded next to the website.</v>
+        <v>Without that the picture is private and residents see a placeholder.</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Leave link blank and the row points at the contact section instead.</v>
+        <v>Paste the ordinary Drive share link. The website converts it itself.</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v/>
+        <v>The section stays hidden until this tab has at least one complete row.</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>ABOUT THE GUIDELINES TAB</v>
+        <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Each rule section is several rows sharing the same 'section' number.</v>
+        <v>ABOUT THE RESOLUTIONS TAB</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Fill in title, keywords and anchor on the FIRST row of a section only.</v>
+        <v>date</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>The 'kind' column decides how the row looks:</v>
+        <v>status</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Passed / Approved / Noted / Deferred / Pending / Rejected — this sets the colour.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>li</v>
+        <v>link</v>
       </c>
       <c r="B52" t="str">
-        <v>a normal bullet point</v>
+        <v>Optional. A link to the full resolution PDF. Leave blank if there isn't one.</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>sub</v>
-      </c>
-      <c r="B53" t="str">
-        <v>a bold sub-heading, e.g. 'Gym' inside the Sports section</v>
+        <v>The 'Latest' button shows the five most recent; 'All' shows everything.</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>note</v>
-      </c>
-      <c r="B54" t="str">
-        <v>a grey highlighted box</v>
+        <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>note-red</v>
-      </c>
-      <c r="B55" t="str">
-        <v>a red warning box</v>
+        <v>ABOUT THE RECORDS TAB</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>note-green</v>
+        <v>type</v>
       </c>
       <c r="B56" t="str">
-        <v>a green box</v>
+        <v>mom = minutes of meeting, notice, or circular. This drives the filter buttons.</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>p</v>
+        <v>date</v>
       </c>
       <c r="B57" t="str">
-        <v>an ordinary paragraph</v>
+        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v/>
+        <v>link</v>
+      </c>
+      <c r="B58" t="str">
+        <v>The PDF file name, e.g. gbm-april-2025.pdf, uploaded next to the website.</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>'keywords' are extra words the website search should match for that section.</v>
+        <v>Leave link blank and the row points at the contact section instead.</v>
       </c>
     </row>
     <row r="60">
@@ -834,32 +836,115 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>IF SOMETHING GOES WRONG</v>
+        <v>ABOUT THE GUIDELINES TAB</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>The website falls back to its built-in copy if this sheet cannot be read,</v>
+        <v>Each rule section is several rows sharing the same 'section' number.</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>so a mistake here can never take the site down. Undo the change and refresh.</v>
+        <v>Fill in title, keywords and anchor on the FIRST row of a section only.</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v/>
+        <v>The 'kind' column decides how the row looks:</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
+        <v>li</v>
+      </c>
+      <c r="B65" t="str">
+        <v>a normal bullet point</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>sub</v>
+      </c>
+      <c r="B66" t="str">
+        <v>a bold sub-heading, e.g. 'Gym' inside the Sports section</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>note</v>
+      </c>
+      <c r="B67" t="str">
+        <v>a grey highlighted box</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>note-red</v>
+      </c>
+      <c r="B68" t="str">
+        <v>a red warning box</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>note-green</v>
+      </c>
+      <c r="B69" t="str">
+        <v>a green box</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>p</v>
+      </c>
+      <c r="B70" t="str">
+        <v>an ordinary paragraph</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>'keywords' are extra words the website search should match for that section.</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>IF SOMETHING GOES WRONG</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>The website falls back to its built-in copy if this sheet cannot be read,</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>so a mistake here can never take the site down. Undo the change and refresh.</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
         <v>Remember: Share -&gt; Anyone with the link -&gt; Viewer, or the website cannot read this.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B65"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B78"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2012,6 +2097,38 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D1"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="13.83203125" customWidth="1"/>
+    <col min="3" max="3" width="64.83203125" customWidth="1"/>
+    <col min="4" max="4" width="52.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" t="str">
+        <v>name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>date</v>
+      </c>
+      <c r="C1" t="str">
+        <v>details</v>
+      </c>
+      <c r="D1" t="str">
+        <v>photo</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D1"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F9"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
@@ -2186,7 +2303,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E9"/>
   <cols>

</xml_diff>

<commit_message>
let the posters come from Google Drive too
The posters tab now takes an ordinary Drive share link in its file column,
the same as the event photographs: the file id is lifted out, rebuilt as a
direct image address, and the other Drive hosts are kept to fall back on.
A plain file name still resolves to images/posters as before.

The retry helper is no longer named after the events section, since the
posters now use it as well.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -435,7 +435,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B78"/>
+  <dimension ref="A1:B79"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="78.83203125" customWidth="1"/>
@@ -649,7 +649,7 @@
         <v>posters</v>
       </c>
       <c r="B32" t="str">
-        <v>Tall 9:16 guideline posters. Use the image file name, or a full https:// link.</v>
+        <v>Tall 9:16 guideline posters. Use a Google Drive link, or the image file name.</v>
       </c>
     </row>
     <row r="33">
@@ -725,7 +725,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>IMPORTANT: each photo in Drive must be shared as</v>
+        <v>IMPORTANT: each picture in Drive must be shared as</v>
       </c>
     </row>
     <row r="44">
@@ -753,198 +753,203 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v/>
+        <v>The posters tab takes Drive links in the same way, with the same sharing rule.</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>ABOUT THE RESOLUTIONS TAB</v>
+        <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>date</v>
-      </c>
-      <c r="B50" t="str">
-        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
+        <v>ABOUT THE RESOLUTIONS TAB</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>status</v>
+        <v>date</v>
       </c>
       <c r="B51" t="str">
-        <v>Passed / Approved / Noted / Deferred / Pending / Rejected — this sets the colour.</v>
+        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>link</v>
+        <v>status</v>
       </c>
       <c r="B52" t="str">
-        <v>Optional. A link to the full resolution PDF. Leave blank if there isn't one.</v>
+        <v>Passed / Approved / Noted / Deferred / Pending / Rejected — this sets the colour.</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>The 'Latest' button shows the five most recent; 'All' shows everything.</v>
+        <v>link</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Optional. A link to the full resolution PDF. Leave blank if there isn't one.</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v/>
+        <v>The 'Latest' button shows the five most recent; 'All' shows everything.</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>ABOUT THE RECORDS TAB</v>
+        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>type</v>
-      </c>
-      <c r="B56" t="str">
-        <v>mom = minutes of meeting, notice, or circular. This drives the filter buttons.</v>
+        <v>ABOUT THE RECORDS TAB</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>date</v>
+        <v>type</v>
       </c>
       <c r="B57" t="str">
-        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
+        <v>mom = minutes of meeting, notice, or circular. This drives the filter buttons.</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>link</v>
+        <v>date</v>
       </c>
       <c r="B58" t="str">
-        <v>The PDF file name, e.g. gbm-april-2025.pdf, uploaded next to the website.</v>
+        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Leave link blank and the row points at the contact section instead.</v>
+        <v>link</v>
+      </c>
+      <c r="B59" t="str">
+        <v>The PDF file name, e.g. gbm-april-2025.pdf, uploaded next to the website.</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v/>
+        <v>Leave link blank and the row points at the contact section instead.</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>ABOUT THE GUIDELINES TAB</v>
+        <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Each rule section is several rows sharing the same 'section' number.</v>
+        <v>ABOUT THE GUIDELINES TAB</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Fill in title, keywords and anchor on the FIRST row of a section only.</v>
+        <v>Each rule section is several rows sharing the same 'section' number.</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>The 'kind' column decides how the row looks:</v>
+        <v>Fill in title, keywords and anchor on the FIRST row of a section only.</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>li</v>
-      </c>
-      <c r="B65" t="str">
-        <v>a normal bullet point</v>
+        <v>The 'kind' column decides how the row looks:</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>sub</v>
+        <v>li</v>
       </c>
       <c r="B66" t="str">
-        <v>a bold sub-heading, e.g. 'Gym' inside the Sports section</v>
+        <v>a normal bullet point</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>note</v>
+        <v>sub</v>
       </c>
       <c r="B67" t="str">
-        <v>a grey highlighted box</v>
+        <v>a bold sub-heading, e.g. 'Gym' inside the Sports section</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>note-red</v>
+        <v>note</v>
       </c>
       <c r="B68" t="str">
-        <v>a red warning box</v>
+        <v>a grey highlighted box</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>note-green</v>
+        <v>note-red</v>
       </c>
       <c r="B69" t="str">
-        <v>a green box</v>
+        <v>a red warning box</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>p</v>
+        <v>note-green</v>
       </c>
       <c r="B70" t="str">
-        <v>an ordinary paragraph</v>
+        <v>a green box</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v/>
+        <v>p</v>
+      </c>
+      <c r="B71" t="str">
+        <v>an ordinary paragraph</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>'keywords' are extra words the website search should match for that section.</v>
+        <v/>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v/>
+        <v>'keywords' are extra words the website search should match for that section.</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>IF SOMETHING GOES WRONG</v>
+        <v/>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>The website falls back to its built-in copy if this sheet cannot be read,</v>
+        <v>IF SOMETHING GOES WRONG</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>so a mistake here can never take the site down. Undo the change and refresh.</v>
+        <v>The website falls back to its built-in copy if this sheet cannot be read,</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v/>
+        <v>so a mistake here can never take the site down. Undo the change and refresh.</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
         <v>Remember: Share -&gt; Anyone with the link -&gt; Viewer, or the website cannot read this.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B78"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B79"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
let the photo gallery come from Google Drive too
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -641,7 +641,7 @@
         <v>gallery</v>
       </c>
       <c r="B31" t="str">
-        <v>Photos. Put the image in the images folder and use its file name in file.</v>
+        <v>Photos. Paste a Google Drive share link in file, or use an images folder file name.</v>
       </c>
     </row>
     <row r="32">
@@ -753,7 +753,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>The posters tab takes Drive links in the same way, with the same sharing rule.</v>
+        <v>The posters and gallery tabs take Drive links in the same way, same sharing rule.</v>
       </c>
     </row>
     <row r="49">

</xml_diff>

<commit_message>
add the improvements tab to the workbook template
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -20,8 +20,9 @@
     <sheet name="gallery" sheetId="15" r:id="rId15"/>
     <sheet name="posters" sheetId="16" r:id="rId16"/>
     <sheet name="events" sheetId="17" r:id="rId17"/>
-    <sheet name="resolutions" sheetId="18" r:id="rId18"/>
-    <sheet name="records" sheetId="19" r:id="rId19"/>
+    <sheet name="improvements" sheetId="18" r:id="rId18"/>
+    <sheet name="resolutions" sheetId="19" r:id="rId19"/>
+    <sheet name="records" sheetId="20" r:id="rId20"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'settings'!A1:B14</definedName>
@@ -40,8 +41,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="14">'gallery'!A1:E9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15">'posters'!A1:C10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16">'events'!A1:D1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17">'resolutions'!A1:F9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18">'records'!A1:E9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17">'improvements'!A1:C17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18">'resolutions'!A1:F9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19">'records'!A1:E9</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -435,7 +437,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B79"/>
+  <dimension ref="A1:B80"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="78.83203125" customWidth="1"/>
@@ -662,294 +664,302 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>resolutions</v>
+        <v>improvements</v>
       </c>
       <c r="B34" t="str">
-        <v>Committee / GBM decisions. Newest first is not required — the site sorts by date.</v>
+        <v>What SSMACS has built since handover. title, category, details. No photo.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>records</v>
+        <v>resolutions</v>
       </c>
       <c r="B35" t="str">
-        <v>Minutes of meetings, notices and circulars. See the note below.</v>
+        <v>Committee / GBM decisions. Newest first is not required — the site sorts by date.</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v/>
+        <v>records</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Minutes of meetings, notices and circulars. See the note below.</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>ABOUT THE EVENTS TAB</v>
+        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>name</v>
-      </c>
-      <c r="B38" t="str">
-        <v>The event, e.g. Ganesh Chaturthi 2026. A row with no name is skipped.</v>
+        <v>ABOUT THE EVENTS TAB</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>date</v>
+        <v>name</v>
       </c>
       <c r="B39" t="str">
-        <v>Type it as 2026-09-14 (year-month-day). The newest event is shown first.</v>
+        <v>The event, e.g. Ganesh Chaturthi 2026. A row with no name is skipped.</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>details</v>
+        <v>date</v>
       </c>
       <c r="B40" t="str">
-        <v>A sentence or two about the day. Optional.</v>
+        <v>Type it as 2026-09-14 (year-month-day). The newest event is shown first.</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>photo</v>
+        <v>details</v>
       </c>
       <c r="B41" t="str">
-        <v>The Google Drive link to the picture. A row with no photo is skipped.</v>
+        <v>A sentence or two about the day. Optional.</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v/>
+        <v>photo</v>
+      </c>
+      <c r="B42" t="str">
+        <v>The Google Drive link to the picture. A row with no photo is skipped.</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>IMPORTANT: each picture in Drive must be shared as</v>
+        <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v/>
-      </c>
-      <c r="B44" t="str">
-        <v>Share -&gt; General access -&gt; Anyone with the link -&gt; Viewer.</v>
+        <v>IMPORTANT: each picture in Drive must be shared as</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Without that the picture is private and residents see a placeholder.</v>
+        <v/>
+      </c>
+      <c r="B45" t="str">
+        <v>Share -&gt; General access -&gt; Anyone with the link -&gt; Viewer.</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Paste the ordinary Drive share link. The website converts it itself.</v>
+        <v>Without that the picture is private and residents see a placeholder.</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>The section stays hidden until this tab has at least one complete row.</v>
+        <v>Paste the ordinary Drive share link. The website converts it itself.</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>The posters and gallery tabs take Drive links in the same way, same sharing rule.</v>
+        <v>The section stays hidden until this tab has at least one complete row.</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v/>
+        <v>The posters and gallery tabs take Drive links in the same way, same sharing rule.</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>ABOUT THE RESOLUTIONS TAB</v>
+        <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>date</v>
-      </c>
-      <c r="B51" t="str">
-        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
+        <v>ABOUT THE RESOLUTIONS TAB</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>status</v>
+        <v>date</v>
       </c>
       <c r="B52" t="str">
-        <v>Passed / Approved / Noted / Deferred / Pending / Rejected — this sets the colour.</v>
+        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>link</v>
+        <v>status</v>
       </c>
       <c r="B53" t="str">
-        <v>Optional. A link to the full resolution PDF. Leave blank if there isn't one.</v>
+        <v>Passed / Approved / Noted / Deferred / Pending / Rejected — this sets the colour.</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>The 'Latest' button shows the five most recent; 'All' shows everything.</v>
+        <v>link</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Optional. A link to the full resolution PDF. Leave blank if there isn't one.</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v/>
+        <v>The 'Latest' button shows the five most recent; 'All' shows everything.</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>ABOUT THE RECORDS TAB</v>
+        <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>type</v>
-      </c>
-      <c r="B57" t="str">
-        <v>mom = minutes of meeting, notice, or circular. This drives the filter buttons.</v>
+        <v>ABOUT THE RECORDS TAB</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>date</v>
+        <v>type</v>
       </c>
       <c r="B58" t="str">
-        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
+        <v>mom = minutes of meeting, notice, or circular. This drives the filter buttons.</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>link</v>
+        <v>date</v>
       </c>
       <c r="B59" t="str">
-        <v>The PDF file name, e.g. gbm-april-2025.pdf, uploaded next to the website.</v>
+        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Leave link blank and the row points at the contact section instead.</v>
+        <v>link</v>
+      </c>
+      <c r="B60" t="str">
+        <v>The PDF file name, e.g. gbm-april-2025.pdf, uploaded next to the website.</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v/>
+        <v>Leave link blank and the row points at the contact section instead.</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>ABOUT THE GUIDELINES TAB</v>
+        <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Each rule section is several rows sharing the same 'section' number.</v>
+        <v>ABOUT THE GUIDELINES TAB</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Fill in title, keywords and anchor on the FIRST row of a section only.</v>
+        <v>Each rule section is several rows sharing the same 'section' number.</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>The 'kind' column decides how the row looks:</v>
+        <v>Fill in title, keywords and anchor on the FIRST row of a section only.</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>li</v>
-      </c>
-      <c r="B66" t="str">
-        <v>a normal bullet point</v>
+        <v>The 'kind' column decides how the row looks:</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>sub</v>
+        <v>li</v>
       </c>
       <c r="B67" t="str">
-        <v>a bold sub-heading, e.g. 'Gym' inside the Sports section</v>
+        <v>a normal bullet point</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>note</v>
+        <v>sub</v>
       </c>
       <c r="B68" t="str">
-        <v>a grey highlighted box</v>
+        <v>a bold sub-heading, e.g. 'Gym' inside the Sports section</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>note-red</v>
+        <v>note</v>
       </c>
       <c r="B69" t="str">
-        <v>a red warning box</v>
+        <v>a grey highlighted box</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>note-green</v>
+        <v>note-red</v>
       </c>
       <c r="B70" t="str">
-        <v>a green box</v>
+        <v>a red warning box</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>p</v>
+        <v>note-green</v>
       </c>
       <c r="B71" t="str">
-        <v>an ordinary paragraph</v>
+        <v>a green box</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v/>
+        <v>p</v>
+      </c>
+      <c r="B72" t="str">
+        <v>an ordinary paragraph</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>'keywords' are extra words the website search should match for that section.</v>
+        <v/>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v/>
+        <v>'keywords' are extra words the website search should match for that section.</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>IF SOMETHING GOES WRONG</v>
+        <v/>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>The website falls back to its built-in copy if this sheet cannot be read,</v>
+        <v>IF SOMETHING GOES WRONG</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>so a mistake here can never take the site down. Undo the change and refresh.</v>
+        <v>The website falls back to its built-in copy if this sheet cannot be read,</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v/>
+        <v>so a mistake here can never take the site down. Undo the change and refresh.</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
         <v>Remember: Share -&gt; Anyone with the link -&gt; Viewer, or the website cannot read this.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B79"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B80"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2134,6 +2144,210 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C17"/>
+  <cols>
+    <col min="1" max="1" width="34.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="64.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" t="str">
+        <v>title</v>
+      </c>
+      <c r="B1" t="str">
+        <v>category</v>
+      </c>
+      <c r="C1" t="str">
+        <v>details</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Amphitheater</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Community spaces</v>
+      </c>
+      <c r="C2" t="str">
+        <v>An open-air stage for gatherings, cultural evenings and religious events.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Kids' play area, badminton &amp; cricket box</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Sports &amp; recreation</v>
+      </c>
+      <c r="C3" t="str">
+        <v>A dedicated play zone for children, with a badminton court and a box cricket area.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Gate 5 opened</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Access &amp; parking</v>
+      </c>
+      <c r="C4" t="str">
+        <v>A new exit gate for the community, easing the load on the existing gates.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Ganesha Temple</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Community spaces</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Built and maintained by the community, with the anniversary celebrated every year.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Security cabins at Gate 1 &amp; Gate 5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Safety &amp; security</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Proper manned cabins, so guards are stationed and sheltered at both gates.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Clear parking demarcation</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Access &amp; parking</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Every bay marked out in hot paint, so allotted parking is unambiguous.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Association office</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Community spaces</v>
+      </c>
+      <c r="C8" t="str">
+        <v>A permanent office for the Association, its records and resident walk-ins.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Yoga room</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Sports &amp; recreation</v>
+      </c>
+      <c r="C9" t="str">
+        <v>A quiet indoor room set aside for yoga and fitness sessions.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Lit walkways through the gardens</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Grounds &amp; landscaping</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Elevated walkways through the planted areas, lit for safe use after dark.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Kitchen area renovated</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Community spaces</v>
+      </c>
+      <c r="C11" t="str">
+        <v>The common kitchen refitted for use during functions and celebrations.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Clean &amp; dry driveways</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Grounds &amp; landscaping</v>
+      </c>
+      <c r="C12" t="str">
+        <v>The garden pipes were concealed to keep the driveway dry and neat.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Fire extinguishers installed</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Safety &amp; security</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Extinguishers fitted across the blocks and the common areas.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Storerooms at multiple locations</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Buildings &amp; utilities</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Secure storage added at several points for equipment and society material.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Swimming pool renovated</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Sports &amp; recreation</v>
+      </c>
+      <c r="C15" t="str">
+        <v>The pool refurbished and brought back into regular use.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Solar fencing restored</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Safety &amp; security</v>
+      </c>
+      <c r="C16" t="str">
+        <v>The perimeter solar fence repaired and made live again.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Cellar water leakage resolved</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Buildings &amp; utilities</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Most of the water leakage issues in the cellars have been resolved.</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C17"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C17"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F9"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
@@ -2304,178 +2518,6 @@
   <autoFilter ref="A1:F9"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
-  <cols>
-    <col min="1" max="1" width="9.83203125" customWidth="1"/>
-    <col min="2" max="2" width="13.83203125" customWidth="1"/>
-    <col min="3" max="3" width="34.83203125" customWidth="1"/>
-    <col min="4" max="4" width="60.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="20" customHeight="1">
-      <c r="A1" t="str">
-        <v>type</v>
-      </c>
-      <c r="B1" t="str">
-        <v>date</v>
-      </c>
-      <c r="C1" t="str">
-        <v>title</v>
-      </c>
-      <c r="D1" t="str">
-        <v>note</v>
-      </c>
-      <c r="E1" t="str">
-        <v>link</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>mom</v>
-      </c>
-      <c r="B2" t="str">
-        <v>2025-04-26</v>
-      </c>
-      <c r="C2" t="str">
-        <v>General Body Meeting — April 2025</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Adoption of Guidelines v1.0, the penalty schedule and the annual accounts.</v>
-      </c>
-      <c r="E2" t="str">
-        <v>#contact</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>notice</v>
-      </c>
-      <c r="B3" t="str">
-        <v>2025-04-02</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Quarterly maintenance due by the 15th</v>
-      </c>
-      <c r="D3" t="str">
-        <v>A 2% per month penalty applies on the outstanding balance after the due date.</v>
-      </c>
-      <c r="E3" t="str">
-        <v>#contact</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>circular</v>
-      </c>
-      <c r="B4" t="str">
-        <v>2025-03-20</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Move-in and move-out timings</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Shifting is permitted only between 9:00 AM and 6:00 PM, with prior intimation to the society office.</v>
-      </c>
-      <c r="E4" t="str">
-        <v>#contact</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>mom</v>
-      </c>
-      <c r="B5" t="str">
-        <v>2025-03-08</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Managing Committee meeting — March 2025</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Penalty schedule finalised, housekeeping review and pool maintenance contract.</v>
-      </c>
-      <c r="E5" t="str">
-        <v>#contact</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>notice</v>
-      </c>
-      <c r="B6" t="str">
-        <v>2025-02-14</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Swimming pool closed every Monday</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Weekly cleaning and water treatment. Normal timings resume on Tuesday.</v>
-      </c>
-      <c r="E6" t="str">
-        <v>#contact</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>mom</v>
-      </c>
-      <c r="B7" t="str">
-        <v>2025-02-01</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Managing Committee meeting — February 2025</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Gate 2 boom barrier rollout, vehicle registration drive and DG maintenance.</v>
-      </c>
-      <c r="E7" t="str">
-        <v>#contact</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>circular</v>
-      </c>
-      <c r="B8" t="str">
-        <v>2025-01-10</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Pet registration and vaccination records</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Pet owners are requested to submit current vaccination certificates to the society office.</v>
-      </c>
-      <c r="E8" t="str">
-        <v>#contact</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>notice</v>
-      </c>
-      <c r="B9" t="str">
-        <v>2024-12-20</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Quiet hours during festive gatherings</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Amplified music is not permitted after 10:00 PM in common areas, as per the guidelines.</v>
-      </c>
-      <c r="E9" t="str">
-        <v>#contact</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:E9"/>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2604,6 +2646,178 @@
   <autoFilter ref="A1:B14"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B14"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E9"/>
+  <cols>
+    <col min="1" max="1" width="9.83203125" customWidth="1"/>
+    <col min="2" max="2" width="13.83203125" customWidth="1"/>
+    <col min="3" max="3" width="34.83203125" customWidth="1"/>
+    <col min="4" max="4" width="60.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" t="str">
+        <v>type</v>
+      </c>
+      <c r="B1" t="str">
+        <v>date</v>
+      </c>
+      <c r="C1" t="str">
+        <v>title</v>
+      </c>
+      <c r="D1" t="str">
+        <v>note</v>
+      </c>
+      <c r="E1" t="str">
+        <v>link</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>mom</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2025-04-26</v>
+      </c>
+      <c r="C2" t="str">
+        <v>General Body Meeting — April 2025</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Adoption of Guidelines v1.0, the penalty schedule and the annual accounts.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>#contact</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>notice</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2025-04-02</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Quarterly maintenance due by the 15th</v>
+      </c>
+      <c r="D3" t="str">
+        <v>A 2% per month penalty applies on the outstanding balance after the due date.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>#contact</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>circular</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2025-03-20</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Move-in and move-out timings</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Shifting is permitted only between 9:00 AM and 6:00 PM, with prior intimation to the society office.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>#contact</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>mom</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2025-03-08</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Managing Committee meeting — March 2025</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Penalty schedule finalised, housekeeping review and pool maintenance contract.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>#contact</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>notice</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2025-02-14</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Swimming pool closed every Monday</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Weekly cleaning and water treatment. Normal timings resume on Tuesday.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>#contact</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>mom</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2025-02-01</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Managing Committee meeting — February 2025</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Gate 2 boom barrier rollout, vehicle registration drive and DG maintenance.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>#contact</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>circular</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2025-01-10</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Pet registration and vaccination records</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Pet owners are requested to submit current vaccination certificates to the society office.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>#contact</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>notice</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2024-12-20</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Quiet hours during festive gatherings</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Amplified music is not permitted after 10:00 PM in common areas, as per the guidelines.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>#contact</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E9"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
add a poster showing how to install the site as an app
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -39,7 +39,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="12">'checklist'!A1:B9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13">'downloads'!A1:C6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14">'gallery'!A1:E9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15">'posters'!A1:C10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15">'posters'!A1:C11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16">'events'!A1:D1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17">'improvements'!A1:C17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18">'resolutions'!A1:F9</definedName>
@@ -1985,7 +1985,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -2005,107 +2005,118 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Balcony safety &amp; cleanliness</v>
+        <v>Add the website to your phone</v>
       </c>
       <c r="B2" t="str">
-        <v>poster-balcony.jpg</v>
+        <v>poster-add-to-home.png</v>
       </c>
       <c r="C2" t="str">
-        <v>Balcony safety &amp; cleanliness — keep your balcony clean and contained, and never throw water, dust, cigarette butts or waste from balconies</v>
+        <v>Add this website to your phone’s home screen and it opens like an app. iPhone: open it in Safari, tap Share, then Add to Home Screen. Android: open it in Chrome, tap the menu, then Add to Home screen. It then works with no signal, opens full screen, keeps every helpline two taps away, and stays up to date on its own.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Corridors must be kept clean &amp; clear</v>
+        <v>Balcony safety &amp; cleanliness</v>
       </c>
       <c r="B3" t="str">
-        <v>poster-corridors.jpg</v>
+        <v>poster-balcony.jpg</v>
       </c>
       <c r="C3" t="str">
-        <v>Corridors must be kept clean &amp; clear — no footwear, cycles, furniture or storage in the common corridors. Keep the passage tidy and unobstructed for everyone.</v>
+        <v>Balcony safety &amp; cleanliness — keep your balcony clean and contained, and never throw water, dust, cigarette butts or waste from balconies</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Parking rules</v>
+        <v>Corridors must be kept clean &amp; clear</v>
       </c>
       <c r="B4" t="str">
-        <v>poster-parking.jpg</v>
+        <v>poster-corridors.jpg</v>
       </c>
       <c r="C4" t="str">
-        <v>Park within your own allotted slot and inside the markings. No-parking zones and fire lanes are strictly enforced — vehicles are locked and fined Rs 200 a day for two-wheelers and Rs 500 for four-wheelers. No waste or storage in parking areas, and cycles belong in flat parking only.</v>
+        <v>Corridors must be kept clean &amp; clear — no footwear, cycles, furniture or storage in the common corridors. Keep the passage tidy and unobstructed for everyone.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Security at the main gate</v>
+        <v>Parking rules</v>
       </c>
       <c r="B5" t="str">
-        <v>poster-gate-security.jpg</v>
+        <v>poster-parking.jpg</v>
       </c>
       <c r="C5" t="str">
-        <v>Residents: affix the society sticker and register your vehicle for automatic access. Guests and non-registered vehicles must use Gate 1 for entry checks. Do not misuse the entry and exit lanes — Gates 3 and 5 are planned for exit only.</v>
+        <v>Park within your own allotted slot and inside the markings. No-parking zones and fire lanes are strictly enforced — vehicles are locked and fined Rs 200 a day for two-wheelers and Rs 500 for four-wheelers. No waste or storage in parking areas, and cycles belong in flat parking only.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Swimming pool usage rules</v>
+        <v>Security at the main gate</v>
       </c>
       <c r="B6" t="str">
-        <v>poster-pool.jpg</v>
+        <v>poster-gate-security.jpg</v>
       </c>
       <c r="C6" t="str">
-        <v>Proper swimwear is mandatory. Children must be supervised by an adult at all times. No food or glass items near the pool. The pool is for registered residents only — guests are not allowed.</v>
+        <v>Residents: affix the society sticker and register your vehicle for automatic access. Guests and non-registered vehicles must use Gate 1 for entry checks. Do not misuse the entry and exit lanes — Gates 3 and 5 are planned for exit only.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Gym guidelines</v>
+        <v>Swimming pool usage rules</v>
       </c>
       <c r="B7" t="str">
-        <v>poster-gym.jpg</v>
+        <v>poster-pool.jpg</v>
       </c>
       <c r="C7" t="str">
-        <v>Under-14s are not allowed in the gym. Do not drop weights or misuse equipment — place them gently and re-rack after use. Limit sessions to 30 minutes during peak hours so everyone gets a chance, and keep the shared audio at a moderate volume.</v>
+        <v>Proper swimwear is mandatory. Children must be supervised by an adult at all times. No food or glass items near the pool. The pool is for registered residents only — guests are not allowed.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Residents’ behaviour towards support staff</v>
+        <v>Gym guidelines</v>
       </c>
       <c r="B8" t="str">
-        <v>poster-staff-behaviour.jpg</v>
+        <v>poster-gym.jpg</v>
       </c>
       <c r="C8" t="str">
-        <v>Treat all support staff with dignity and courtesy — a smile and kind words go a long way. Do not be rude, dismissive or abusive towards support staff; mistreating them creates an unhealthy environment and is serious misconduct.</v>
+        <v>Under-14s are not allowed in the gym. Do not drop weights or misuse equipment — place them gently and re-rack after use. Limit sessions to 30 minutes during peak hours so everyone gets a chance, and keep the shared audio at a moderate volume.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Resident &amp; support staff interaction</v>
+        <v>Residents’ behaviour towards support staff</v>
       </c>
       <c r="B9" t="str">
-        <v>poster-staff-interaction.jpg</v>
+        <v>poster-staff-behaviour.jpg</v>
       </c>
       <c r="C9" t="str">
-        <v>Support staff are valued members of our society’s ecosystem and courteous interaction is expected at all times. They may not be engaged for private work inside flats beyond their defined scope. Verbal abuse, intimidation or disrespectful behaviour is strictly unacceptable — report any misconduct to the Maintenance Manager or Core Committee.</v>
+        <v>Treat all support staff with dignity and courtesy — a smile and kind words go a long way. Do not be rude, dismissive or abusive towards support staff; mistreating them creates an unhealthy environment and is serious misconduct.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
+        <v>Resident &amp; support staff interaction</v>
+      </c>
+      <c r="B10" t="str">
+        <v>poster-staff-interaction.jpg</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Support staff are valued members of our society’s ecosystem and courteous interaction is expected at all times. They may not be engaged for private work inside flats beyond their defined scope. Verbal abuse, intimidation or disrespectful behaviour is strictly unacceptable — report any misconduct to the Maintenance Manager or Core Committee.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v>Save water — use it judiciously</v>
       </c>
-      <c r="B10" t="str">
+      <c r="B11" t="str">
         <v>poster-savewater.png</v>
       </c>
-      <c r="C10" t="str">
+      <c r="C11" t="str">
         <v>Boond boond se banta hai kal ka savera. Close taps when not in use, use a bucket instead of a shower, run full loads in washing machines, report leaks promptly, and water plants in the morning or evening.</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C10"/>
+  <autoFilter ref="A1:C11"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
announce the resident portal launch on the first poster
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -2005,13 +2005,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Add the website to your phone</v>
+        <v>Our Resident Information Portal is live</v>
       </c>
       <c r="B2" t="str">
-        <v>poster-add-to-home.png</v>
+        <v>poster-portal-launch.png</v>
       </c>
       <c r="C2" t="str">
-        <v>Add this website to your phone’s home screen and it opens like an app. iPhone: open it in Safari, tap Share, then Add to Home Screen. Android: open it in Chrome, tap the menu, then Add to Home screen. It then works with no signal, opens full screen, keeps every helpline two taps away, and stays up to date on its own.</v>
+        <v>Our Resident Information Portal is now live at shwetashubham.netlify.app — the society guidelines in full with a search box, amenity timings, helpline numbers you can tap to call, the approved fees and penalty schedule, the committee directory, meeting minutes, notices and resolutions, these posters and the new resident checklist. No login, no app store, no charge. Add it to your home screen and it opens like an app, readable even with no signal.</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
show the year beside each improvement
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -41,7 +41,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="14">'gallery'!A1:E9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15">'posters'!A1:C11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16">'events'!A1:D1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17">'improvements'!A1:C17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17">'improvements'!A1:D19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18">'resolutions'!A1:F9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19">'records'!A1:E9</definedName>
   </definedNames>
@@ -667,7 +667,7 @@
         <v>improvements</v>
       </c>
       <c r="B34" t="str">
-        <v>What SSMACS has built since handover. title, category, details. No photo.</v>
+        <v>What SSMACS has built since handover. title, category, year, details. No photo.</v>
       </c>
     </row>
     <row r="35">
@@ -2155,11 +2155,12 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:D19"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="64.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="64.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -2170,6 +2171,9 @@
         <v>category</v>
       </c>
       <c r="C1" t="str">
+        <v>year</v>
+      </c>
+      <c r="D1" t="str">
         <v>details</v>
       </c>
     </row>
@@ -2178,181 +2182,257 @@
         <v>Amphitheater</v>
       </c>
       <c r="B2" t="str">
-        <v>Community spaces</v>
+        <v>Community Spaces</v>
       </c>
       <c r="C2" t="str">
-        <v>An open-air stage for gatherings, cultural evenings and religious events.</v>
+        <v>2024</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Open-air stage created for community gatherings, cultural programs and religious events.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Kids' play area, badminton &amp; cricket box</v>
+        <v>Ganesha Temple</v>
       </c>
       <c r="B3" t="str">
-        <v>Sports &amp; recreation</v>
+        <v>Community Spaces</v>
       </c>
       <c r="C3" t="str">
-        <v>A dedicated play zone for children, with a badminton court and a box cricket area.</v>
+        <v>2024</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Temple constructed and maintained by the community, with its anniversary celebrated annually.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Gate 5 opened</v>
+        <v>Association Office</v>
       </c>
       <c r="B4" t="str">
-        <v>Access &amp; parking</v>
+        <v>Community Spaces</v>
       </c>
       <c r="C4" t="str">
-        <v>A new exit gate for the community, easing the load on the existing gates.</v>
+        <v>2024</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Permanent office established for Association operations, records and resident interactions.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Ganesha Temple</v>
+        <v>Kitchen Area Renovation</v>
       </c>
       <c r="B5" t="str">
-        <v>Community spaces</v>
+        <v>Community Spaces</v>
       </c>
       <c r="C5" t="str">
-        <v>Built and maintained by the community, with the anniversary celebrated every year.</v>
+        <v>2024</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Common kitchen renovated to support community functions, celebrations and events.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Security cabins at Gate 1 &amp; Gate 5</v>
+        <v>Swimming Pool Renovation</v>
       </c>
       <c r="B6" t="str">
-        <v>Safety &amp; security</v>
+        <v>Sports &amp; Recreation</v>
       </c>
       <c r="C6" t="str">
-        <v>Proper manned cabins, so guards are stationed and sheltered at both gates.</v>
+        <v>2024</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Swimming pool refurbished and restored for regular use.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Clear parking demarcation</v>
+        <v>Solar Fencing Restoration</v>
       </c>
       <c r="B7" t="str">
-        <v>Access &amp; parking</v>
+        <v>Safety &amp; Security</v>
       </c>
       <c r="C7" t="str">
-        <v>Every bay marked out in hot paint, so allotted parking is unambiguous.</v>
+        <v>2024</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Perimeter solar fencing repaired and restored to working condition.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Association office</v>
+        <v>Cellar Water Leakage Resolution</v>
       </c>
       <c r="B8" t="str">
-        <v>Community spaces</v>
+        <v>Buildings &amp; Utilities</v>
       </c>
       <c r="C8" t="str">
-        <v>A permanent office for the Association, its records and resident walk-ins.</v>
+        <v>2024</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Majority of cellar water-leakage issues addressed and resolved.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Yoga room</v>
+        <v>Clean &amp; Dry Driveways</v>
       </c>
       <c r="B9" t="str">
-        <v>Sports &amp; recreation</v>
+        <v>Grounds &amp; Landscaping</v>
       </c>
       <c r="C9" t="str">
-        <v>A quiet indoor room set aside for yoga and fitness sessions.</v>
+        <v>2024</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Garden water pipes concealed to prevent water on driveways and improve overall appearance.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Lit walkways through the gardens</v>
+        <v>Kids’ Play Area, Badminton &amp; Box Cricket</v>
       </c>
       <c r="B10" t="str">
-        <v>Grounds &amp; landscaping</v>
+        <v>Sports &amp; Recreation</v>
       </c>
       <c r="C10" t="str">
-        <v>Elevated walkways through the planted areas, lit for safe use after dark.</v>
+        <v>2025</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Dedicated children’s play area, badminton court and box-cricket facility created.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Kitchen area renovated</v>
+        <v>Yoga Room</v>
       </c>
       <c r="B11" t="str">
-        <v>Community spaces</v>
+        <v>Sports &amp; Recreation</v>
       </c>
       <c r="C11" t="str">
-        <v>The common kitchen refitted for use during functions and celebrations.</v>
+        <v>2025</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Dedicated indoor space created for yoga, fitness and wellness activities.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Clean &amp; dry driveways</v>
+        <v>Gate 5 Opening</v>
       </c>
       <c r="B12" t="str">
-        <v>Grounds &amp; landscaping</v>
+        <v>Access &amp; Parking</v>
       </c>
       <c r="C12" t="str">
-        <v>The garden pipes were concealed to keep the driveway dry and neat.</v>
+        <v>2025</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Additional community exit opened to improve access and reduce load on existing gates.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Fire extinguishers installed</v>
+        <v>Security Cabins – Gates 1 &amp; 5</v>
       </c>
       <c r="B13" t="str">
-        <v>Safety &amp; security</v>
+        <v>Safety &amp; Security</v>
       </c>
       <c r="C13" t="str">
-        <v>Extinguishers fitted across the blocks and the common areas.</v>
+        <v>2025</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Permanent sheltered security cabins established at both gates.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Storerooms at multiple locations</v>
+        <v>Parking Demarcation</v>
       </c>
       <c r="B14" t="str">
-        <v>Buildings &amp; utilities</v>
+        <v>Access &amp; Parking</v>
       </c>
       <c r="C14" t="str">
-        <v>Secure storage added at several points for equipment and society material.</v>
+        <v>2025</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Parking bays clearly marked using hot paint to ensure unambiguous allocation.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Swimming pool renovated</v>
+        <v>Fire Extinguishers</v>
       </c>
       <c r="B15" t="str">
-        <v>Sports &amp; recreation</v>
+        <v>Safety &amp; Security</v>
       </c>
       <c r="C15" t="str">
-        <v>The pool refurbished and brought back into regular use.</v>
+        <v>2025</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Fire extinguishers installed across residential blocks and common areas.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Solar fencing restored</v>
+        <v>Multiple Storerooms</v>
       </c>
       <c r="B16" t="str">
-        <v>Safety &amp; security</v>
+        <v>Buildings &amp; Utilities</v>
       </c>
       <c r="C16" t="str">
-        <v>The perimeter solar fence repaired and made live again.</v>
+        <v>2025</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Secure storage spaces created at multiple locations for society equipment and materials.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Cellar water leakage resolved</v>
+        <v>Automated Number Plate Recognition (ANPR) Boom Barrier</v>
       </c>
       <c r="B17" t="str">
-        <v>Buildings &amp; utilities</v>
+        <v>Safety, Security &amp; Access</v>
       </c>
       <c r="C17" t="str">
-        <v>Most of the water leakage issues in the cellars have been resolved.</v>
+        <v>2025</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Modern automated boom barrier with number-plate recognition introduced to strengthen vehicle access control and improve entry/exit management.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>New Snooker &amp; Carrom Facilities</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Sports &amp; Recreation</v>
+      </c>
+      <c r="C18" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D18" t="str">
+        <v>New snooker table and carrom board added to enhance indoor recreational facilities for residents.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Garden Walkways with Lighting</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Grounds &amp; Landscaping</v>
+      </c>
+      <c r="C19" t="str">
+        <v>2026</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Elevated walkways created through landscaped areas with lighting for safe evening use.</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C17"/>
+  <autoFilter ref="A1:D19"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D19"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
let an event be a film as well as a photograph
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -40,7 +40,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="13">'downloads'!A1:C6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14">'gallery'!A1:E9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15">'posters'!A1:C11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16">'events'!A1:D1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16">'events'!A1:E1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17">'improvements'!A1:D19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18">'resolutions'!A1:F9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19">'records'!A1:E9</definedName>
@@ -437,7 +437,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B80"/>
+  <dimension ref="A1:B84"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="78.83203125" customWidth="1"/>
@@ -725,226 +725,229 @@
         <v>photo</v>
       </c>
       <c r="B42" t="str">
-        <v>The Google Drive link to the picture. A row with no photo is skipped.</v>
+        <v>The Google Drive link to the picture. Leave blank if the row has a video.</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v/>
+        <v>video</v>
+      </c>
+      <c r="B43" t="str">
+        <v>The Google Drive link to a video, or a YouTube link. Optional.</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>IMPORTANT: each picture in Drive must be shared as</v>
+        <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v/>
-      </c>
-      <c r="B45" t="str">
-        <v>Share -&gt; General access -&gt; Anyone with the link -&gt; Viewer.</v>
+        <v>A row needs a name and either a photo or a video. A video slide shows a still</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Without that the picture is private and residents see a placeholder.</v>
+        <v>from the film with a play button; tapping it plays the film full screen.</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Paste the ordinary Drive share link. The website converts it itself.</v>
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>The section stays hidden until this tab has at least one complete row.</v>
+        <v>IMPORTANT: each picture in Drive must be shared as</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>The posters and gallery tabs take Drive links in the same way, same sharing rule.</v>
+        <v/>
+      </c>
+      <c r="B49" t="str">
+        <v>Share -&gt; General access -&gt; Anyone with the link -&gt; Viewer.</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v/>
+        <v>Without that the picture is private and residents see a placeholder.</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>ABOUT THE RESOLUTIONS TAB</v>
+        <v>Paste the ordinary Drive share link. The website converts it itself.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>date</v>
-      </c>
-      <c r="B52" t="str">
-        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
+        <v>The section stays hidden until this tab has at least one complete row.</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>status</v>
-      </c>
-      <c r="B53" t="str">
-        <v>Passed / Approved / Noted / Deferred / Pending / Rejected — this sets the colour.</v>
+        <v>The posters and gallery tabs take Drive links in the same way, same sharing rule.</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>link</v>
-      </c>
-      <c r="B54" t="str">
-        <v>Optional. A link to the full resolution PDF. Leave blank if there isn't one.</v>
+        <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>The 'Latest' button shows the five most recent; 'All' shows everything.</v>
+        <v>ABOUT THE RESOLUTIONS TAB</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v/>
+        <v>date</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>ABOUT THE RECORDS TAB</v>
+        <v>status</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Passed / Approved / Noted / Deferred / Pending / Rejected — this sets the colour.</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>type</v>
+        <v>link</v>
       </c>
       <c r="B58" t="str">
-        <v>mom = minutes of meeting, notice, or circular. This drives the filter buttons.</v>
+        <v>Optional. A link to the full resolution PDF. Leave blank if there isn't one.</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>date</v>
-      </c>
-      <c r="B59" t="str">
-        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
+        <v>The 'Latest' button shows the five most recent; 'All' shows everything.</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>link</v>
-      </c>
-      <c r="B60" t="str">
-        <v>The PDF file name, e.g. gbm-april-2025.pdf, uploaded next to the website.</v>
+        <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Leave link blank and the row points at the contact section instead.</v>
+        <v>ABOUT THE RECORDS TAB</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v/>
+        <v>type</v>
+      </c>
+      <c r="B62" t="str">
+        <v>mom = minutes of meeting, notice, or circular. This drives the filter buttons.</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>ABOUT THE GUIDELINES TAB</v>
+        <v>date</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Each rule section is several rows sharing the same 'section' number.</v>
+        <v>link</v>
+      </c>
+      <c r="B64" t="str">
+        <v>The PDF file name, e.g. gbm-april-2025.pdf, uploaded next to the website.</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Fill in title, keywords and anchor on the FIRST row of a section only.</v>
+        <v>Leave link blank and the row points at the contact section instead.</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>The 'kind' column decides how the row looks:</v>
+        <v/>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>li</v>
-      </c>
-      <c r="B67" t="str">
-        <v>a normal bullet point</v>
+        <v>ABOUT THE GUIDELINES TAB</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>sub</v>
-      </c>
-      <c r="B68" t="str">
-        <v>a bold sub-heading, e.g. 'Gym' inside the Sports section</v>
+        <v>Each rule section is several rows sharing the same 'section' number.</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>note</v>
-      </c>
-      <c r="B69" t="str">
-        <v>a grey highlighted box</v>
+        <v>Fill in title, keywords and anchor on the FIRST row of a section only.</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>note-red</v>
-      </c>
-      <c r="B70" t="str">
-        <v>a red warning box</v>
+        <v>The 'kind' column decides how the row looks:</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>note-green</v>
+        <v>li</v>
       </c>
       <c r="B71" t="str">
-        <v>a green box</v>
+        <v>a normal bullet point</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>p</v>
+        <v>sub</v>
       </c>
       <c r="B72" t="str">
-        <v>an ordinary paragraph</v>
+        <v>a bold sub-heading, e.g. 'Gym' inside the Sports section</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v/>
+        <v>note</v>
+      </c>
+      <c r="B73" t="str">
+        <v>a grey highlighted box</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>'keywords' are extra words the website search should match for that section.</v>
+        <v>note-red</v>
+      </c>
+      <c r="B74" t="str">
+        <v>a red warning box</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v/>
+        <v>note-green</v>
+      </c>
+      <c r="B75" t="str">
+        <v>a green box</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>IF SOMETHING GOES WRONG</v>
+        <v>p</v>
+      </c>
+      <c r="B76" t="str">
+        <v>an ordinary paragraph</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>The website falls back to its built-in copy if this sheet cannot be read,</v>
+        <v/>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>so a mistake here can never take the site down. Undo the change and refresh.</v>
+        <v>'keywords' are extra words the website search should match for that section.</v>
       </c>
     </row>
     <row r="79">
@@ -954,12 +957,32 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
+        <v>IF SOMETHING GOES WRONG</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>The website falls back to its built-in copy if this sheet cannot be read,</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>so a mistake here can never take the site down. Undo the change and refresh.</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
         <v>Remember: Share -&gt; Anyone with the link -&gt; Viewer, or the website cannot read this.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B80"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B84"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2123,12 +2146,13 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="13.83203125" customWidth="1"/>
     <col min="3" max="3" width="64.83203125" customWidth="1"/>
     <col min="4" max="4" width="52.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -2144,11 +2168,14 @@
       <c r="D1" t="str">
         <v>photo</v>
       </c>
+      <c r="E1" t="str">
+        <v>video</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D1"/>
+  <autoFilter ref="A1:E1"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
link the guidelines to the copy kept in Google Drive
The committee keeps the signed PDF in the society Drive, so the download now
points there and the file can be replaced without redeploying the site. Any
link beginning http is opened in a new tab, since a cross-origin download
attribute is ignored anyway and navigating away would lose the resident's
place. The PDF beside index.html stays as the backup.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -635,7 +635,7 @@
         <v>downloads</v>
       </c>
       <c r="B30" t="str">
-        <v>Forms and documents. Put the file next to the website and use its file name in url.</v>
+        <v>Forms and documents. Paste a Google Drive share link in url, or a file name kept beside the website.</v>
       </c>
     </row>
     <row r="31">
@@ -1776,10 +1776,10 @@
         <v>Society Guidelines (PDF)</v>
       </c>
       <c r="B2" t="str">
-        <v>Version 1.0 · Approved in the April GBM</v>
+        <v>Version 1.0 · Approved in the April GBM · opens in Google Drive</v>
       </c>
       <c r="C2" t="str">
-        <v>Shweta-Shubham-Guidelines.pdf</v>
+        <v>https://drive.google.com/file/d/1mVuDWy87M-03UZk2oDmKb6ewWdaRcH_k/view</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
name the section Infrastructure & Facilities Created by SSMACS
The committee asked for the fuller wording in place of 'Built since handover',
and for the association to be written SSMACS throughout — the guidelines
footer had it as SSMAC. The footer link keeps a short form so the column
still reads cleanly.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -667,7 +667,7 @@
         <v>improvements</v>
       </c>
       <c r="B34" t="str">
-        <v>What SSMACS has built since handover. title, category, year, details. No photo.</v>
+        <v>Infrastructure and facilities created by SSMACS. title, category, year, details. No photo.</v>
       </c>
     </row>
     <row r="35">
@@ -2749,7 +2749,7 @@
         <v>footer_note</v>
       </c>
       <c r="B13" t="str">
-        <v>Guidelines v1.0 · Prepared by SSMAC · Approved in the April GBM</v>
+        <v>Guidelines v1.0 · Prepared by SSMACS · Approved in the April GBM</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
say it plainly on the poster: the portal fits in your pocket
The committee wanted the one-tap, keep-it-on-your-phone idea said up front
rather than left to the panel near the bottom, so the headline strapline,
the home-screen panel and the caption all carry it now.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -2028,13 +2028,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Our Resident Information Portal is live</v>
+        <v>The portal, in your pocket – in one tap</v>
       </c>
       <c r="B2" t="str">
         <v>poster-portal-launch.png</v>
       </c>
       <c r="C2" t="str">
-        <v>Our Resident Information Portal is now live at shwetashubham.in — the society guidelines in full with a search box, amenity timings, helpline numbers you can tap to call, the approved fees and penalty schedule, the committee directory, meeting minutes, notices and resolutions, these posters and the new resident checklist. No login, no app store, no charge. Add it to your home screen and it opens like an app, readable even with no signal.</v>
+        <v>Our Resident Information Portal is now live at shwetashubham.in — everything about the society in your pocket. The guidelines in full with a search box, amenity timings, helpline numbers you can tap to call, the approved fees and penalty schedule, the committee directory, meeting minutes, notices and resolutions, these posters and the new resident checklist. No login, no app store, no charge. One tap adds it to your home screen, where it opens like an app and stays readable even with no signal.</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
publish the gate access timings
Residents are turned away at a closed gate at night and have no way to check
which one is open, so the notice now sits on the page under the timings
quick-reference. A gate's periods are written as separate rows and joined
into one cell, the way the printed notice reads, and a period worded exactly
Closed is shown as a red badge so a shut gate is obvious at a glance.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -10,19 +10,20 @@
     <sheet name="quick_actions" sheetId="5" r:id="rId5"/>
     <sheet name="helplines" sheetId="6" r:id="rId6"/>
     <sheet name="timings" sheetId="7" r:id="rId7"/>
-    <sheet name="guidelines" sheetId="8" r:id="rId8"/>
-    <sheet name="staff_scope" sheetId="9" r:id="rId9"/>
-    <sheet name="fees" sheetId="10" r:id="rId10"/>
-    <sheet name="committee" sheetId="11" r:id="rId11"/>
-    <sheet name="escalation" sheetId="12" r:id="rId12"/>
-    <sheet name="checklist" sheetId="13" r:id="rId13"/>
-    <sheet name="downloads" sheetId="14" r:id="rId14"/>
-    <sheet name="gallery" sheetId="15" r:id="rId15"/>
-    <sheet name="posters" sheetId="16" r:id="rId16"/>
-    <sheet name="events" sheetId="17" r:id="rId17"/>
-    <sheet name="improvements" sheetId="18" r:id="rId18"/>
-    <sheet name="resolutions" sheetId="19" r:id="rId19"/>
-    <sheet name="records" sheetId="20" r:id="rId20"/>
+    <sheet name="gates" sheetId="8" r:id="rId8"/>
+    <sheet name="guidelines" sheetId="9" r:id="rId9"/>
+    <sheet name="staff_scope" sheetId="10" r:id="rId10"/>
+    <sheet name="fees" sheetId="11" r:id="rId11"/>
+    <sheet name="committee" sheetId="12" r:id="rId12"/>
+    <sheet name="escalation" sheetId="13" r:id="rId13"/>
+    <sheet name="checklist" sheetId="14" r:id="rId14"/>
+    <sheet name="downloads" sheetId="15" r:id="rId15"/>
+    <sheet name="gallery" sheetId="16" r:id="rId16"/>
+    <sheet name="posters" sheetId="17" r:id="rId17"/>
+    <sheet name="events" sheetId="18" r:id="rId18"/>
+    <sheet name="improvements" sheetId="19" r:id="rId19"/>
+    <sheet name="resolutions" sheetId="20" r:id="rId20"/>
+    <sheet name="records" sheetId="21" r:id="rId21"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'settings'!A1:B14</definedName>
@@ -31,19 +32,20 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4">'quick_actions'!A1:D11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5">'helplines'!A1:E12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6">'timings'!A1:C11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7">'guidelines'!A1:F139</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8">'staff_scope'!A1:D37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9">'fees'!A1:E17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10">'committee'!A1:F21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11">'escalation'!A1:C5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12">'checklist'!A1:B9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13">'downloads'!A1:C6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14">'gallery'!A1:E9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15">'posters'!A1:C11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16">'events'!A1:E1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17">'improvements'!A1:D19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18">'resolutions'!A1:F9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="19">'records'!A1:E9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7">'gates'!A1:C10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8">'guidelines'!A1:F139</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9">'staff_scope'!A1:D37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10">'fees'!A1:E17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11">'committee'!A1:F21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12">'escalation'!A1:C5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13">'checklist'!A1:B9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14">'downloads'!A1:C6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15">'gallery'!A1:E9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16">'posters'!A1:C11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17">'events'!A1:E1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18">'improvements'!A1:D19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19">'resolutions'!A1:F9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20">'records'!A1:E9</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -437,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B84"/>
+  <dimension ref="A1:B85"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="78.83203125" customWidth="1"/>
@@ -616,378 +618,922 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>escalation</v>
+        <v>gates</v>
       </c>
       <c r="B28" t="str">
-        <v>Who to contact, in order</v>
+        <v>Which gate is open, when, and to whom. Repeat the gate name on each of its rows.</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>checklist</v>
+        <v>escalation</v>
       </c>
       <c r="B29" t="str">
-        <v>The new-resident checklist. Numbering is automatic.</v>
+        <v>Who to contact, in order</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>downloads</v>
+        <v>checklist</v>
       </c>
       <c r="B30" t="str">
-        <v>Forms and documents. Paste a Google Drive share link in url, or a file name kept beside the website.</v>
+        <v>The new-resident checklist. Numbering is automatic.</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>gallery</v>
+        <v>downloads</v>
       </c>
       <c r="B31" t="str">
-        <v>Photos. Paste a Google Drive share link in file, or use an images folder file name.</v>
+        <v>Forms and documents. Paste a Google Drive share link in url, or a file name kept beside the website.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>posters</v>
+        <v>gallery</v>
       </c>
       <c r="B32" t="str">
-        <v>Tall 9:16 guideline posters. Use a Google Drive link, or the image file name.</v>
+        <v>Photos. Paste a Google Drive share link in file, or use an images folder file name.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>events</v>
+        <v>posters</v>
       </c>
       <c r="B33" t="str">
-        <v>Photographs from society events. See the note below.</v>
+        <v>Tall 9:16 guideline posters. Use a Google Drive link, or the image file name.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>improvements</v>
+        <v>events</v>
       </c>
       <c r="B34" t="str">
-        <v>Infrastructure and facilities created by SSMACS. title, category, year, details. No photo.</v>
+        <v>Photographs from society events. See the note below.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>resolutions</v>
+        <v>improvements</v>
       </c>
       <c r="B35" t="str">
-        <v>Committee / GBM decisions. Newest first is not required — the site sorts by date.</v>
+        <v>Infrastructure and facilities created by SSMACS. title, category, year, details. No photo.</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>records</v>
+        <v>resolutions</v>
       </c>
       <c r="B36" t="str">
-        <v>Minutes of meetings, notices and circulars. See the note below.</v>
+        <v>Committee / GBM decisions. Newest first is not required — the site sorts by date.</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v/>
+        <v>records</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Minutes of meetings, notices and circulars. See the note below.</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>ABOUT THE EVENTS TAB</v>
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>name</v>
-      </c>
-      <c r="B39" t="str">
-        <v>The event, e.g. Ganesh Chaturthi 2026. A row with no name is skipped.</v>
+        <v>ABOUT THE EVENTS TAB</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>date</v>
+        <v>name</v>
       </c>
       <c r="B40" t="str">
-        <v>Type it as 2026-09-14 (year-month-day). The newest event is shown first.</v>
+        <v>The event, e.g. Ganesh Chaturthi 2026. A row with no name is skipped.</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>details</v>
+        <v>date</v>
       </c>
       <c r="B41" t="str">
-        <v>A sentence or two about the day. Optional.</v>
+        <v>Type it as 2026-09-14 (year-month-day). The newest event is shown first.</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>photo</v>
+        <v>details</v>
       </c>
       <c r="B42" t="str">
-        <v>The Google Drive link to the picture. Leave blank if the row has a video.</v>
+        <v>A sentence or two about the day. Optional.</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>video</v>
+        <v>photo</v>
       </c>
       <c r="B43" t="str">
-        <v>The Google Drive link to a video, or a YouTube link. Optional.</v>
+        <v>The Google Drive link to the picture. Leave blank if the row has a video.</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v/>
+        <v>video</v>
+      </c>
+      <c r="B44" t="str">
+        <v>The Google Drive link to a video, or a YouTube link. Optional.</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>A row needs a name and either a photo or a video. A video slide shows a still</v>
+        <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>from the film with a play button; tapping it plays the film full screen.</v>
+        <v>A row needs a name and either a photo or a video. A video slide shows a still</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v/>
+        <v>from the film with a play button; tapping it plays the film full screen.</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>IMPORTANT: each picture in Drive must be shared as</v>
+        <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v/>
-      </c>
-      <c r="B49" t="str">
-        <v>Share -&gt; General access -&gt; Anyone with the link -&gt; Viewer.</v>
+        <v>IMPORTANT: each picture in Drive must be shared as</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Without that the picture is private and residents see a placeholder.</v>
+        <v/>
+      </c>
+      <c r="B50" t="str">
+        <v>Share -&gt; General access -&gt; Anyone with the link -&gt; Viewer.</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Paste the ordinary Drive share link. The website converts it itself.</v>
+        <v>Without that the picture is private and residents see a placeholder.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>The section stays hidden until this tab has at least one complete row.</v>
+        <v>Paste the ordinary Drive share link. The website converts it itself.</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>The posters and gallery tabs take Drive links in the same way, same sharing rule.</v>
+        <v>The section stays hidden until this tab has at least one complete row.</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v/>
+        <v>The posters and gallery tabs take Drive links in the same way, same sharing rule.</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>ABOUT THE RESOLUTIONS TAB</v>
+        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>date</v>
-      </c>
-      <c r="B56" t="str">
-        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
+        <v>ABOUT THE RESOLUTIONS TAB</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>status</v>
+        <v>date</v>
       </c>
       <c r="B57" t="str">
-        <v>Passed / Approved / Noted / Deferred / Pending / Rejected — this sets the colour.</v>
+        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>link</v>
+        <v>status</v>
       </c>
       <c r="B58" t="str">
-        <v>Optional. A link to the full resolution PDF. Leave blank if there isn't one.</v>
+        <v>Passed / Approved / Noted / Deferred / Pending / Rejected — this sets the colour.</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>The 'Latest' button shows the five most recent; 'All' shows everything.</v>
+        <v>link</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Optional. A link to the full resolution PDF. Leave blank if there isn't one.</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v/>
+        <v>The 'Latest' button shows the five most recent; 'All' shows everything.</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>ABOUT THE RECORDS TAB</v>
+        <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>type</v>
-      </c>
-      <c r="B62" t="str">
-        <v>mom = minutes of meeting, notice, or circular. This drives the filter buttons.</v>
+        <v>ABOUT THE RECORDS TAB</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>date</v>
+        <v>type</v>
       </c>
       <c r="B63" t="str">
-        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
+        <v>mom = minutes of meeting, notice, or circular. This drives the filter buttons.</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>link</v>
+        <v>date</v>
       </c>
       <c r="B64" t="str">
-        <v>The PDF file name, e.g. gbm-april-2025.pdf, uploaded next to the website.</v>
+        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Leave link blank and the row points at the contact section instead.</v>
+        <v>link</v>
+      </c>
+      <c r="B65" t="str">
+        <v>The PDF file name, e.g. gbm-april-2025.pdf, uploaded next to the website.</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v/>
+        <v>Leave link blank and the row points at the contact section instead.</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>ABOUT THE GUIDELINES TAB</v>
+        <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Each rule section is several rows sharing the same 'section' number.</v>
+        <v>ABOUT THE GUIDELINES TAB</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Fill in title, keywords and anchor on the FIRST row of a section only.</v>
+        <v>Each rule section is several rows sharing the same 'section' number.</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>The 'kind' column decides how the row looks:</v>
+        <v>Fill in title, keywords and anchor on the FIRST row of a section only.</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>li</v>
-      </c>
-      <c r="B71" t="str">
-        <v>a normal bullet point</v>
+        <v>The 'kind' column decides how the row looks:</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>sub</v>
+        <v>li</v>
       </c>
       <c r="B72" t="str">
-        <v>a bold sub-heading, e.g. 'Gym' inside the Sports section</v>
+        <v>a normal bullet point</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>note</v>
+        <v>sub</v>
       </c>
       <c r="B73" t="str">
-        <v>a grey highlighted box</v>
+        <v>a bold sub-heading, e.g. 'Gym' inside the Sports section</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>note-red</v>
+        <v>note</v>
       </c>
       <c r="B74" t="str">
-        <v>a red warning box</v>
+        <v>a grey highlighted box</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>note-green</v>
+        <v>note-red</v>
       </c>
       <c r="B75" t="str">
-        <v>a green box</v>
+        <v>a red warning box</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>p</v>
+        <v>note-green</v>
       </c>
       <c r="B76" t="str">
-        <v>an ordinary paragraph</v>
+        <v>a green box</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v/>
+        <v>p</v>
+      </c>
+      <c r="B77" t="str">
+        <v>an ordinary paragraph</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>'keywords' are extra words the website search should match for that section.</v>
+        <v/>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v/>
+        <v>'keywords' are extra words the website search should match for that section.</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>IF SOMETHING GOES WRONG</v>
+        <v/>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>The website falls back to its built-in copy if this sheet cannot be read,</v>
+        <v>IF SOMETHING GOES WRONG</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>so a mistake here can never take the site down. Undo the change and refresh.</v>
+        <v>The website falls back to its built-in copy if this sheet cannot be read,</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v/>
+        <v>so a mistake here can never take the site down. Undo the change and refresh.</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
         <v>Remember: Share -&gt; Anyone with the link -&gt; Viewer, or the website cannot read this.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B84"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B85"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D37"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="6.83203125" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" customWidth="1"/>
+    <col min="4" max="4" width="90.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" t="str">
+        <v>role</v>
+      </c>
+      <c r="B1" t="str">
+        <v>icon</v>
+      </c>
+      <c r="C1" t="str">
+        <v>group</v>
+      </c>
+      <c r="D1" t="str">
+        <v>text</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Electrician</v>
+      </c>
+      <c r="B2" t="str">
+        <v>⚡</v>
+      </c>
+      <c r="C2" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Common area electrical infrastructure — corridor and cellar lights, lift power supply, DG connections, motor panels</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Electrician</v>
+      </c>
+      <c r="B3" t="str">
+        <v>⚡</v>
+      </c>
+      <c r="C3" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Faults up to the flat's MCB point</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Electrician</v>
+      </c>
+      <c r="B4" t="str">
+        <v>⚡</v>
+      </c>
+      <c r="C4" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Periodic inspection of panels, switchboards and DG wiring</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Electrician</v>
+      </c>
+      <c r="B5" t="str">
+        <v>⚡</v>
+      </c>
+      <c r="C5" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D5" t="str">
+        <v>DG operations during power outages</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Electrician</v>
+      </c>
+      <c r="B6" t="str">
+        <v>⚡</v>
+      </c>
+      <c r="C6" t="str">
+        <v>not_covered</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Any electrical work inside flats beyond the MCB point</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Electrician</v>
+      </c>
+      <c r="B7" t="str">
+        <v>⚡</v>
+      </c>
+      <c r="C7" t="str">
+        <v>not_covered</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Personal appliances, fixtures or internal wiring</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Electrician</v>
+      </c>
+      <c r="B8" t="str">
+        <v>⚡</v>
+      </c>
+      <c r="C8" t="str">
+        <v>not_covered</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Engage your own licensed electrician</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Plumber</v>
+      </c>
+      <c r="B9" t="str">
+        <v>🚰</v>
+      </c>
+      <c r="C9" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D9" t="str">
+        <v>WTP, STP, drainage systems and overhead water tanks</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Plumber</v>
+      </c>
+      <c r="B10" t="str">
+        <v>🚰</v>
+      </c>
+      <c r="C10" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Water levels, pump operations and pipelines across the society</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Plumber</v>
+      </c>
+      <c r="B11" t="str">
+        <v>🚰</v>
+      </c>
+      <c r="C11" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Cellar drainage, rainwater harvesting and external pipeline repairs</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Plumber</v>
+      </c>
+      <c r="B12" t="str">
+        <v>🚰</v>
+      </c>
+      <c r="C12" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Leakages and blockages inside flats on a best-effort basis during working hours</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Plumber</v>
+      </c>
+      <c r="B13" t="str">
+        <v>🚰</v>
+      </c>
+      <c r="C13" t="str">
+        <v>not_covered</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Tap repairs, faucet replacements or fixture installation inside flats</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Plumber</v>
+      </c>
+      <c r="B14" t="str">
+        <v>🚰</v>
+      </c>
+      <c r="C14" t="str">
+        <v>not_covered</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Internal bathroom or kitchen plumbing modifications and renovations</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Plumber</v>
+      </c>
+      <c r="B15" t="str">
+        <v>🚰</v>
+      </c>
+      <c r="C15" t="str">
+        <v>not_covered</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Engage your own licensed plumber</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Housekeeping</v>
+      </c>
+      <c r="B16" t="str">
+        <v>🧹</v>
+      </c>
+      <c r="C16" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Corridors, staircases, lobbies, lifts, reception and clubhouse</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Housekeeping</v>
+      </c>
+      <c r="B17" t="str">
+        <v>🧹</v>
+      </c>
+      <c r="C17" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Gym, pool surroundings, indoor games room, yoga room, amphitheater</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Housekeeping</v>
+      </c>
+      <c r="B18" t="str">
+        <v>🧹</v>
+      </c>
+      <c r="C18" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Guest rooms, including bedsheets and towels between bookings</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Housekeeping</v>
+      </c>
+      <c r="B19" t="str">
+        <v>🧹</v>
+      </c>
+      <c r="C19" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Cellars, parking areas, driveways, ducts and cobweb cleaning</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Housekeeping</v>
+      </c>
+      <c r="B20" t="str">
+        <v>🧹</v>
+      </c>
+      <c r="C20" t="str">
+        <v>not_covered</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Cleaning or domestic work inside individual flats</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Housekeeping</v>
+      </c>
+      <c r="B21" t="str">
+        <v>🧹</v>
+      </c>
+      <c r="C21" t="str">
+        <v>not_covered</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Personal errands, grocery carrying or shifting assistance</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Gardener</v>
+      </c>
+      <c r="B22" t="str">
+        <v>🌱</v>
+      </c>
+      <c r="C22" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Lawns, flower beds, hedges, potted plants and tree lines in common areas</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Gardener</v>
+      </c>
+      <c r="B23" t="str">
+        <v>🌱</v>
+      </c>
+      <c r="C23" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Watering, pruning, trimming and seasonal planting</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Gardener</v>
+      </c>
+      <c r="B24" t="str">
+        <v>🌱</v>
+      </c>
+      <c r="C24" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Tot-lot greens, walkway plants and entrance landscaping</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Gardener</v>
+      </c>
+      <c r="B25" t="str">
+        <v>🌱</v>
+      </c>
+      <c r="C25" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Fertilisers, pesticides and soil treatment for common greenery</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Gardener</v>
+      </c>
+      <c r="B26" t="str">
+        <v>🌱</v>
+      </c>
+      <c r="C26" t="str">
+        <v>not_covered</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Gardening inside flats, balconies or terraces</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Gardener</v>
+      </c>
+      <c r="B27" t="str">
+        <v>🌱</v>
+      </c>
+      <c r="C27" t="str">
+        <v>not_covered</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Personal plant purchases, potting or balcony garden setup</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Security Personnel</v>
+      </c>
+      <c r="B28" t="str">
+        <v>🛡</v>
+      </c>
+      <c r="C28" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Check-in and check-out of all persons and vehicles at entry and exit gates</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Security Personnel</v>
+      </c>
+      <c r="B29" t="str">
+        <v>🛡</v>
+      </c>
+      <c r="C29" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Visitor identity verification and the visitor register</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Security Personnel</v>
+      </c>
+      <c r="B30" t="str">
+        <v>🛡</v>
+      </c>
+      <c r="C30" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Vehicle movement log and gate entry process</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Security Personnel</v>
+      </c>
+      <c r="B31" t="str">
+        <v>🛡</v>
+      </c>
+      <c r="C31" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D31" t="str">
+        <v>First response to fire and medical emergencies outside working hours</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Security Personnel</v>
+      </c>
+      <c r="B32" t="str">
+        <v>🛡</v>
+      </c>
+      <c r="C32" t="str">
+        <v>covered</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Periodic night rounds of cellars, corridors and common areas</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Security Personnel</v>
+      </c>
+      <c r="B33" t="str">
+        <v>🛡</v>
+      </c>
+      <c r="C33" t="str">
+        <v>duties</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Cooperate with entry and exit checks without exception</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Security Personnel</v>
+      </c>
+      <c r="B34" t="str">
+        <v>🛡</v>
+      </c>
+      <c r="C34" t="str">
+        <v>duties</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Pre-inform about large gatherings or external visitors</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Security Personnel</v>
+      </c>
+      <c r="B35" t="str">
+        <v>🛡</v>
+      </c>
+      <c r="C35" t="str">
+        <v>duties</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Do not assign security staff tasks outside their duties</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Treat staff with respect</v>
+      </c>
+      <c r="B36" t="str">
+        <v>👤</v>
+      </c>
+      <c r="C36" t="str">
+        <v>prose</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Support staff are valued members of our society's ecosystem, working to ensure a safe and comfortable living environment for everyone. Courteous and respectful interaction is expected at all times.</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Treat staff with respect</v>
+      </c>
+      <c r="B37" t="str">
+        <v>👤</v>
+      </c>
+      <c r="C37" t="str">
+        <v>prose</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Any form of verbal abuse, intimidation or disrespectful behaviour towards support staff is strictly unacceptable and may be escalated to the Core Committee. Complaints about staff should be reported to the Maintenance Manager or Core Committee.</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D37"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D37"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E17"/>
   <cols>
@@ -1217,7 +1763,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F21"/>
   <cols>
@@ -1591,7 +2137,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C5"/>
   <cols>
@@ -1663,7 +2209,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B9"/>
   <cols>
@@ -1751,7 +2297,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C6"/>
   <cols>
@@ -1834,7 +2380,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E9"/>
   <cols>
@@ -2006,7 +2552,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C11"/>
   <cols>
@@ -2144,7 +2690,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E1"/>
   <cols>
@@ -2180,7 +2726,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D19"/>
   <cols>
@@ -2460,182 +3006,6 @@
   <autoFilter ref="A1:D19"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:D19"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F9"/>
-  <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="13.83203125" customWidth="1"/>
-    <col min="3" max="3" width="34.83203125" customWidth="1"/>
-    <col min="4" max="4" width="70.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="20" customHeight="1">
-      <c r="A1" t="str">
-        <v>ref</v>
-      </c>
-      <c r="B1" t="str">
-        <v>date</v>
-      </c>
-      <c r="C1" t="str">
-        <v>title</v>
-      </c>
-      <c r="D1" t="str">
-        <v>summary</v>
-      </c>
-      <c r="E1" t="str">
-        <v>status</v>
-      </c>
-      <c r="F1" t="str">
-        <v>link</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>GBM/2025/01</v>
-      </c>
-      <c r="B2" t="str">
-        <v>2025-04-26</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Society Guidelines v1.0 adopted</v>
-      </c>
-      <c r="D2" t="str">
-        <v>The consolidated guidelines document was approved and circulated to all owners and tenants for sign-off.</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>MC/2025/04</v>
-      </c>
-      <c r="B3" t="str">
-        <v>2025-03-12</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Penalty schedule for guideline violations</v>
-      </c>
-      <c r="D3" t="str">
-        <v>A consolidated schedule of fines was approved, to be applied uniformly across all blocks.</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>MC/2025/03</v>
-      </c>
-      <c r="B4" t="str">
-        <v>2025-02-08</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Quarterly maintenance due on the 15th</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Maintenance is payable quarterly through NoBrokerhood, with a 2% per month penalty on overdue balances.</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>MC/2025/02</v>
-      </c>
-      <c r="B5" t="str">
-        <v>2025-01-18</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Swimming pool closed on Mondays</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Weekly cleaning and water treatment scheduled for Mondays; normal timings resume Tuesday.</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>MC/2025/01</v>
-      </c>
-      <c r="B6" t="str">
-        <v>2025-01-04</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Vehicle registration for Gate 2 access</v>
-      </c>
-      <c r="D6" t="str">
-        <v>All resident vehicles must be registered with the society office for boom barrier access at Gate 2.</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>GBM/2024/02</v>
-      </c>
-      <c r="B7" t="str">
-        <v>2024-12-15</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Housekeeping and security agency appointment</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Appointment of the housekeeping and security agencies for the following financial year was ratified.</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>MC/2024/07</v>
-      </c>
-      <c r="B8" t="str">
-        <v>2024-11-09</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Clubhouse and guest room booking rules</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Bookings are first-come, first-served through the Maintenance Manager, with charges as per the fee schedule.</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>MC/2024/06</v>
-      </c>
-      <c r="B9" t="str">
-        <v>2024-09-21</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Festival celebrations and volunteer participation</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Celebrations remain optional and subject to resident participation, volunteer availability and committee approval.</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Noted</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:F9"/>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2769,6 +3139,182 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F9"/>
+  <cols>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="13.83203125" customWidth="1"/>
+    <col min="3" max="3" width="34.83203125" customWidth="1"/>
+    <col min="4" max="4" width="70.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" t="str">
+        <v>ref</v>
+      </c>
+      <c r="B1" t="str">
+        <v>date</v>
+      </c>
+      <c r="C1" t="str">
+        <v>title</v>
+      </c>
+      <c r="D1" t="str">
+        <v>summary</v>
+      </c>
+      <c r="E1" t="str">
+        <v>status</v>
+      </c>
+      <c r="F1" t="str">
+        <v>link</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>GBM/2025/01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2025-04-26</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Society Guidelines v1.0 adopted</v>
+      </c>
+      <c r="D2" t="str">
+        <v>The consolidated guidelines document was approved and circulated to all owners and tenants for sign-off.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>MC/2025/04</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2025-03-12</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Penalty schedule for guideline violations</v>
+      </c>
+      <c r="D3" t="str">
+        <v>A consolidated schedule of fines was approved, to be applied uniformly across all blocks.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>MC/2025/03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2025-02-08</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Quarterly maintenance due on the 15th</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Maintenance is payable quarterly through NoBrokerhood, with a 2% per month penalty on overdue balances.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>MC/2025/02</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2025-01-18</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Swimming pool closed on Mondays</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Weekly cleaning and water treatment scheduled for Mondays; normal timings resume Tuesday.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>MC/2025/01</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2025-01-04</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Vehicle registration for Gate 2 access</v>
+      </c>
+      <c r="D6" t="str">
+        <v>All resident vehicles must be registered with the society office for boom barrier access at Gate 2.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>GBM/2024/02</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2024-12-15</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Housekeeping and security agency appointment</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Appointment of the housekeeping and security agencies for the following financial year was ratified.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>MC/2024/07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2024-11-09</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Clubhouse and guest room booking rules</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Bookings are first-come, first-served through the Maintenance Manager, with charges as per the fee schedule.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>MC/2024/06</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2024-09-21</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Festival celebrations and volunteer participation</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Celebrations remain optional and subject to resident participation, volunteer availability and committee approval.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Noted</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F9"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E9"/>
   <cols>
@@ -3682,6 +4228,133 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C10"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" t="str">
+        <v>gate</v>
+      </c>
+      <c r="B1" t="str">
+        <v>timing</v>
+      </c>
+      <c r="C1" t="str">
+        <v>access</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>**Gate 1**</v>
+      </c>
+      <c r="B2" t="str">
+        <v>6:00 AM – 11:00 PM</v>
+      </c>
+      <c r="C2" t="str">
+        <v>**Guests &amp; vendors – entry &amp; exit**</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>**Gate 1**</v>
+      </c>
+      <c r="B3" t="str">
+        <v>11:00 PM – 6:00 AM</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Closed</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>**Gate 2**</v>
+      </c>
+      <c r="B4" t="str">
+        <v>6:00 AM – 11:00 PM</v>
+      </c>
+      <c r="C4" t="str">
+        <v>**Owners – entry only**</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>**Gate 2**</v>
+      </c>
+      <c r="B5" t="str">
+        <v>11:00 PM – 6:00 AM</v>
+      </c>
+      <c r="C5" t="str">
+        <v>**Entry &amp; exit – all vehicles**</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>**Gate 3**</v>
+      </c>
+      <c r="B6" t="str">
+        <v>6:00 AM – 11:00 PM</v>
+      </c>
+      <c r="C6" t="str">
+        <v>**Exit only**</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>**Gate 3**</v>
+      </c>
+      <c r="B7" t="str">
+        <v>11:00 PM – 6:00 AM</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Closed</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>**Gate 4**</v>
+      </c>
+      <c r="B8" t="str">
+        <v>All day</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Closed</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>**Gate 5**</v>
+      </c>
+      <c r="B9" t="str">
+        <v>6:00 AM – 11:00 PM</v>
+      </c>
+      <c r="C9" t="str">
+        <v>**Exit only**</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>**Gate 5**</v>
+      </c>
+      <c r="B10" t="str">
+        <v>11:00 PM – 6:00 AM</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Closed</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C10"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C10"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F139"/>
   <cols>
     <col min="1" max="1" width="9.83203125" customWidth="1"/>
@@ -5311,540 +5984,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:F139"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D37"/>
-  <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="6.83203125" customWidth="1"/>
-    <col min="3" max="3" width="13.83203125" customWidth="1"/>
-    <col min="4" max="4" width="90.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="20" customHeight="1">
-      <c r="A1" t="str">
-        <v>role</v>
-      </c>
-      <c r="B1" t="str">
-        <v>icon</v>
-      </c>
-      <c r="C1" t="str">
-        <v>group</v>
-      </c>
-      <c r="D1" t="str">
-        <v>text</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Electrician</v>
-      </c>
-      <c r="B2" t="str">
-        <v>⚡</v>
-      </c>
-      <c r="C2" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Common area electrical infrastructure — corridor and cellar lights, lift power supply, DG connections, motor panels</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Electrician</v>
-      </c>
-      <c r="B3" t="str">
-        <v>⚡</v>
-      </c>
-      <c r="C3" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Faults up to the flat's MCB point</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Electrician</v>
-      </c>
-      <c r="B4" t="str">
-        <v>⚡</v>
-      </c>
-      <c r="C4" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Periodic inspection of panels, switchboards and DG wiring</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Electrician</v>
-      </c>
-      <c r="B5" t="str">
-        <v>⚡</v>
-      </c>
-      <c r="C5" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D5" t="str">
-        <v>DG operations during power outages</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Electrician</v>
-      </c>
-      <c r="B6" t="str">
-        <v>⚡</v>
-      </c>
-      <c r="C6" t="str">
-        <v>not_covered</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Any electrical work inside flats beyond the MCB point</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Electrician</v>
-      </c>
-      <c r="B7" t="str">
-        <v>⚡</v>
-      </c>
-      <c r="C7" t="str">
-        <v>not_covered</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Personal appliances, fixtures or internal wiring</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Electrician</v>
-      </c>
-      <c r="B8" t="str">
-        <v>⚡</v>
-      </c>
-      <c r="C8" t="str">
-        <v>not_covered</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Engage your own licensed electrician</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Plumber</v>
-      </c>
-      <c r="B9" t="str">
-        <v>🚰</v>
-      </c>
-      <c r="C9" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D9" t="str">
-        <v>WTP, STP, drainage systems and overhead water tanks</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Plumber</v>
-      </c>
-      <c r="B10" t="str">
-        <v>🚰</v>
-      </c>
-      <c r="C10" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Water levels, pump operations and pipelines across the society</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Plumber</v>
-      </c>
-      <c r="B11" t="str">
-        <v>🚰</v>
-      </c>
-      <c r="C11" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Cellar drainage, rainwater harvesting and external pipeline repairs</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Plumber</v>
-      </c>
-      <c r="B12" t="str">
-        <v>🚰</v>
-      </c>
-      <c r="C12" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Leakages and blockages inside flats on a best-effort basis during working hours</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Plumber</v>
-      </c>
-      <c r="B13" t="str">
-        <v>🚰</v>
-      </c>
-      <c r="C13" t="str">
-        <v>not_covered</v>
-      </c>
-      <c r="D13" t="str">
-        <v>Tap repairs, faucet replacements or fixture installation inside flats</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Plumber</v>
-      </c>
-      <c r="B14" t="str">
-        <v>🚰</v>
-      </c>
-      <c r="C14" t="str">
-        <v>not_covered</v>
-      </c>
-      <c r="D14" t="str">
-        <v>Internal bathroom or kitchen plumbing modifications and renovations</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Plumber</v>
-      </c>
-      <c r="B15" t="str">
-        <v>🚰</v>
-      </c>
-      <c r="C15" t="str">
-        <v>not_covered</v>
-      </c>
-      <c r="D15" t="str">
-        <v>Engage your own licensed plumber</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Housekeeping</v>
-      </c>
-      <c r="B16" t="str">
-        <v>🧹</v>
-      </c>
-      <c r="C16" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D16" t="str">
-        <v>Corridors, staircases, lobbies, lifts, reception and clubhouse</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>Housekeeping</v>
-      </c>
-      <c r="B17" t="str">
-        <v>🧹</v>
-      </c>
-      <c r="C17" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D17" t="str">
-        <v>Gym, pool surroundings, indoor games room, yoga room, amphitheater</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>Housekeeping</v>
-      </c>
-      <c r="B18" t="str">
-        <v>🧹</v>
-      </c>
-      <c r="C18" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D18" t="str">
-        <v>Guest rooms, including bedsheets and towels between bookings</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>Housekeeping</v>
-      </c>
-      <c r="B19" t="str">
-        <v>🧹</v>
-      </c>
-      <c r="C19" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D19" t="str">
-        <v>Cellars, parking areas, driveways, ducts and cobweb cleaning</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>Housekeeping</v>
-      </c>
-      <c r="B20" t="str">
-        <v>🧹</v>
-      </c>
-      <c r="C20" t="str">
-        <v>not_covered</v>
-      </c>
-      <c r="D20" t="str">
-        <v>Cleaning or domestic work inside individual flats</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>Housekeeping</v>
-      </c>
-      <c r="B21" t="str">
-        <v>🧹</v>
-      </c>
-      <c r="C21" t="str">
-        <v>not_covered</v>
-      </c>
-      <c r="D21" t="str">
-        <v>Personal errands, grocery carrying or shifting assistance</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>Gardener</v>
-      </c>
-      <c r="B22" t="str">
-        <v>🌱</v>
-      </c>
-      <c r="C22" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D22" t="str">
-        <v>Lawns, flower beds, hedges, potted plants and tree lines in common areas</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>Gardener</v>
-      </c>
-      <c r="B23" t="str">
-        <v>🌱</v>
-      </c>
-      <c r="C23" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D23" t="str">
-        <v>Watering, pruning, trimming and seasonal planting</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>Gardener</v>
-      </c>
-      <c r="B24" t="str">
-        <v>🌱</v>
-      </c>
-      <c r="C24" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D24" t="str">
-        <v>Tot-lot greens, walkway plants and entrance landscaping</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>Gardener</v>
-      </c>
-      <c r="B25" t="str">
-        <v>🌱</v>
-      </c>
-      <c r="C25" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D25" t="str">
-        <v>Fertilisers, pesticides and soil treatment for common greenery</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>Gardener</v>
-      </c>
-      <c r="B26" t="str">
-        <v>🌱</v>
-      </c>
-      <c r="C26" t="str">
-        <v>not_covered</v>
-      </c>
-      <c r="D26" t="str">
-        <v>Gardening inside flats, balconies or terraces</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>Gardener</v>
-      </c>
-      <c r="B27" t="str">
-        <v>🌱</v>
-      </c>
-      <c r="C27" t="str">
-        <v>not_covered</v>
-      </c>
-      <c r="D27" t="str">
-        <v>Personal plant purchases, potting or balcony garden setup</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>Security Personnel</v>
-      </c>
-      <c r="B28" t="str">
-        <v>🛡</v>
-      </c>
-      <c r="C28" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D28" t="str">
-        <v>Check-in and check-out of all persons and vehicles at entry and exit gates</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>Security Personnel</v>
-      </c>
-      <c r="B29" t="str">
-        <v>🛡</v>
-      </c>
-      <c r="C29" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D29" t="str">
-        <v>Visitor identity verification and the visitor register</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>Security Personnel</v>
-      </c>
-      <c r="B30" t="str">
-        <v>🛡</v>
-      </c>
-      <c r="C30" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D30" t="str">
-        <v>Vehicle movement log and gate entry process</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>Security Personnel</v>
-      </c>
-      <c r="B31" t="str">
-        <v>🛡</v>
-      </c>
-      <c r="C31" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D31" t="str">
-        <v>First response to fire and medical emergencies outside working hours</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>Security Personnel</v>
-      </c>
-      <c r="B32" t="str">
-        <v>🛡</v>
-      </c>
-      <c r="C32" t="str">
-        <v>covered</v>
-      </c>
-      <c r="D32" t="str">
-        <v>Periodic night rounds of cellars, corridors and common areas</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>Security Personnel</v>
-      </c>
-      <c r="B33" t="str">
-        <v>🛡</v>
-      </c>
-      <c r="C33" t="str">
-        <v>duties</v>
-      </c>
-      <c r="D33" t="str">
-        <v>Cooperate with entry and exit checks without exception</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>Security Personnel</v>
-      </c>
-      <c r="B34" t="str">
-        <v>🛡</v>
-      </c>
-      <c r="C34" t="str">
-        <v>duties</v>
-      </c>
-      <c r="D34" t="str">
-        <v>Pre-inform about large gatherings or external visitors</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>Security Personnel</v>
-      </c>
-      <c r="B35" t="str">
-        <v>🛡</v>
-      </c>
-      <c r="C35" t="str">
-        <v>duties</v>
-      </c>
-      <c r="D35" t="str">
-        <v>Do not assign security staff tasks outside their duties</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>Treat staff with respect</v>
-      </c>
-      <c r="B36" t="str">
-        <v>👤</v>
-      </c>
-      <c r="C36" t="str">
-        <v>prose</v>
-      </c>
-      <c r="D36" t="str">
-        <v>Support staff are valued members of our society's ecosystem, working to ensure a safe and comfortable living environment for everyone. Courteous and respectful interaction is expected at all times.</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>Treat staff with respect</v>
-      </c>
-      <c r="B37" t="str">
-        <v>👤</v>
-      </c>
-      <c r="C37" t="str">
-        <v>prose</v>
-      </c>
-      <c r="D37" t="str">
-        <v>Any form of verbal abuse, intimidation or disrespectful behaviour towards support staff is strictly unacceptable and may be escalated to the Core Committee. Complaints about staff should be reported to the Maintenance Manager or Core Committee.</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:D37"/>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D37"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
show residents the icon they will end up with
The poster asked people to add the portal to their home screen without ever
showing them what that looks like, so it now carries a phone with the icon
sitting on a home screen, named, next to the written steps.

The launch notice also had to be pinned. Posters are driven by the sheet, and
the sheet replaced the whole row of them, so the announcement was being wiped
off the live page the moment the posters tab loaded.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -41,7 +41,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="13">'checklist'!A1:B9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14">'downloads'!A1:C6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15">'gallery'!A1:E9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16">'posters'!A1:C11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16">'posters'!A1:C10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17">'events'!A1:E1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18">'improvements'!A1:D19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19">'resolutions'!A1:F9</definedName>
@@ -2554,7 +2554,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C10"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -2574,118 +2574,107 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>The portal, in your pocket – in one tap</v>
+        <v>Balcony safety &amp; cleanliness</v>
       </c>
       <c r="B2" t="str">
-        <v>poster-portal-launch.png</v>
+        <v>poster-balcony.jpg</v>
       </c>
       <c r="C2" t="str">
-        <v>Our Resident Information Portal is now live at shwetashubham.in — everything about the society in your pocket. The guidelines in full with a search box, amenity timings, helpline numbers you can tap to call, the approved fees and penalty schedule, the committee directory, meeting minutes, notices and resolutions, these posters and the new resident checklist. No login, no app store, no charge. One tap adds it to your home screen, where it opens like an app and stays readable even with no signal.</v>
+        <v>Balcony safety &amp; cleanliness — keep your balcony clean and contained, and never throw water, dust, cigarette butts or waste from balconies</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Balcony safety &amp; cleanliness</v>
+        <v>Corridors must be kept clean &amp; clear</v>
       </c>
       <c r="B3" t="str">
-        <v>poster-balcony.jpg</v>
+        <v>poster-corridors.jpg</v>
       </c>
       <c r="C3" t="str">
-        <v>Balcony safety &amp; cleanliness — keep your balcony clean and contained, and never throw water, dust, cigarette butts or waste from balconies</v>
+        <v>Corridors must be kept clean &amp; clear — no footwear, cycles, furniture or storage in the common corridors. Keep the passage tidy and unobstructed for everyone.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Corridors must be kept clean &amp; clear</v>
+        <v>Parking rules</v>
       </c>
       <c r="B4" t="str">
-        <v>poster-corridors.jpg</v>
+        <v>poster-parking.jpg</v>
       </c>
       <c r="C4" t="str">
-        <v>Corridors must be kept clean &amp; clear — no footwear, cycles, furniture or storage in the common corridors. Keep the passage tidy and unobstructed for everyone.</v>
+        <v>Park within your own allotted slot and inside the markings. No-parking zones and fire lanes are strictly enforced — vehicles are locked and fined Rs 200 a day for two-wheelers and Rs 500 for four-wheelers. No waste or storage in parking areas, and cycles belong in flat parking only.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Parking rules</v>
+        <v>Security at the main gate</v>
       </c>
       <c r="B5" t="str">
-        <v>poster-parking.jpg</v>
+        <v>poster-gate-security.jpg</v>
       </c>
       <c r="C5" t="str">
-        <v>Park within your own allotted slot and inside the markings. No-parking zones and fire lanes are strictly enforced — vehicles are locked and fined Rs 200 a day for two-wheelers and Rs 500 for four-wheelers. No waste or storage in parking areas, and cycles belong in flat parking only.</v>
+        <v>Residents: affix the society sticker and register your vehicle for automatic access. Guests and non-registered vehicles must use Gate 1 for entry checks. Do not misuse the entry and exit lanes — Gates 3 and 5 are planned for exit only.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Security at the main gate</v>
+        <v>Swimming pool usage rules</v>
       </c>
       <c r="B6" t="str">
-        <v>poster-gate-security.jpg</v>
+        <v>poster-pool.jpg</v>
       </c>
       <c r="C6" t="str">
-        <v>Residents: affix the society sticker and register your vehicle for automatic access. Guests and non-registered vehicles must use Gate 1 for entry checks. Do not misuse the entry and exit lanes — Gates 3 and 5 are planned for exit only.</v>
+        <v>Proper swimwear is mandatory. Children must be supervised by an adult at all times. No food or glass items near the pool. The pool is for registered residents only — guests are not allowed.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Swimming pool usage rules</v>
+        <v>Gym guidelines</v>
       </c>
       <c r="B7" t="str">
-        <v>poster-pool.jpg</v>
+        <v>poster-gym.jpg</v>
       </c>
       <c r="C7" t="str">
-        <v>Proper swimwear is mandatory. Children must be supervised by an adult at all times. No food or glass items near the pool. The pool is for registered residents only — guests are not allowed.</v>
+        <v>Under-14s are not allowed in the gym. Do not drop weights or misuse equipment — place them gently and re-rack after use. Limit sessions to 30 minutes during peak hours so everyone gets a chance, and keep the shared audio at a moderate volume.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Gym guidelines</v>
+        <v>Residents’ behaviour towards support staff</v>
       </c>
       <c r="B8" t="str">
-        <v>poster-gym.jpg</v>
+        <v>poster-staff-behaviour.jpg</v>
       </c>
       <c r="C8" t="str">
-        <v>Under-14s are not allowed in the gym. Do not drop weights or misuse equipment — place them gently and re-rack after use. Limit sessions to 30 minutes during peak hours so everyone gets a chance, and keep the shared audio at a moderate volume.</v>
+        <v>Treat all support staff with dignity and courtesy — a smile and kind words go a long way. Do not be rude, dismissive or abusive towards support staff; mistreating them creates an unhealthy environment and is serious misconduct.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Residents’ behaviour towards support staff</v>
+        <v>Resident &amp; support staff interaction</v>
       </c>
       <c r="B9" t="str">
-        <v>poster-staff-behaviour.jpg</v>
+        <v>poster-staff-interaction.jpg</v>
       </c>
       <c r="C9" t="str">
-        <v>Treat all support staff with dignity and courtesy — a smile and kind words go a long way. Do not be rude, dismissive or abusive towards support staff; mistreating them creates an unhealthy environment and is serious misconduct.</v>
+        <v>Support staff are valued members of our society’s ecosystem and courteous interaction is expected at all times. They may not be engaged for private work inside flats beyond their defined scope. Verbal abuse, intimidation or disrespectful behaviour is strictly unacceptable — report any misconduct to the Maintenance Manager or Core Committee.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Resident &amp; support staff interaction</v>
+        <v>Save water — use it judiciously</v>
       </c>
       <c r="B10" t="str">
-        <v>poster-staff-interaction.jpg</v>
+        <v>poster-savewater.png</v>
       </c>
       <c r="C10" t="str">
-        <v>Support staff are valued members of our society’s ecosystem and courteous interaction is expected at all times. They may not be engaged for private work inside flats beyond their defined scope. Verbal abuse, intimidation or disrespectful behaviour is strictly unacceptable — report any misconduct to the Maintenance Manager or Core Committee.</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Save water — use it judiciously</v>
-      </c>
-      <c r="B11" t="str">
-        <v>poster-savewater.png</v>
-      </c>
-      <c r="C11" t="str">
         <v>Boond boond se banta hai kal ka savera. Close taps when not in use, use a bucket instead of a shower, run full loads in washing machines, report leaks promptly, and water plants in the morning or evening.</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C11"/>
+  <autoFilter ref="A1:C10"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C10"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
let the sheet own the posters outright
Pinning the launch notice into the page meant one poster the committee could
not reorder or retire from the sheet. The posters tab is now the whole list
again, and the launch poster is just another row they can add, move or drop.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -41,7 +41,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="13">'checklist'!A1:B9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14">'downloads'!A1:C6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15">'gallery'!A1:E9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16">'posters'!A1:C10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16">'posters'!A1:C11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17">'events'!A1:E1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18">'improvements'!A1:D19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19">'resolutions'!A1:F9</definedName>
@@ -2554,7 +2554,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -2574,107 +2574,118 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Balcony safety &amp; cleanliness</v>
+        <v>The portal, in your pocket – in one tap</v>
       </c>
       <c r="B2" t="str">
-        <v>poster-balcony.jpg</v>
+        <v>poster-portal-launch.png</v>
       </c>
       <c r="C2" t="str">
-        <v>Balcony safety &amp; cleanliness — keep your balcony clean and contained, and never throw water, dust, cigarette butts or waste from balconies</v>
+        <v>Our Resident Information Portal is now live at shwetashubham.in — everything about the society in your pocket. The guidelines in full with a search box, amenity timings, helpline numbers you can tap to call, the approved fees and penalty schedule, the committee directory, meeting minutes, notices and resolutions, these posters and the new resident checklist. No login, no app store, no charge. One tap adds it to your home screen, where it opens like an app and stays readable even with no signal. The phone in the picture shows exactly how the icon will look once you have added it.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Corridors must be kept clean &amp; clear</v>
+        <v>Balcony safety &amp; cleanliness</v>
       </c>
       <c r="B3" t="str">
-        <v>poster-corridors.jpg</v>
+        <v>poster-balcony.jpg</v>
       </c>
       <c r="C3" t="str">
-        <v>Corridors must be kept clean &amp; clear — no footwear, cycles, furniture or storage in the common corridors. Keep the passage tidy and unobstructed for everyone.</v>
+        <v>Balcony safety &amp; cleanliness — keep your balcony clean and contained, and never throw water, dust, cigarette butts or waste from balconies</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Parking rules</v>
+        <v>Corridors must be kept clean &amp; clear</v>
       </c>
       <c r="B4" t="str">
-        <v>poster-parking.jpg</v>
+        <v>poster-corridors.jpg</v>
       </c>
       <c r="C4" t="str">
-        <v>Park within your own allotted slot and inside the markings. No-parking zones and fire lanes are strictly enforced — vehicles are locked and fined Rs 200 a day for two-wheelers and Rs 500 for four-wheelers. No waste or storage in parking areas, and cycles belong in flat parking only.</v>
+        <v>Corridors must be kept clean &amp; clear — no footwear, cycles, furniture or storage in the common corridors. Keep the passage tidy and unobstructed for everyone.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Security at the main gate</v>
+        <v>Parking rules</v>
       </c>
       <c r="B5" t="str">
-        <v>poster-gate-security.jpg</v>
+        <v>poster-parking.jpg</v>
       </c>
       <c r="C5" t="str">
-        <v>Residents: affix the society sticker and register your vehicle for automatic access. Guests and non-registered vehicles must use Gate 1 for entry checks. Do not misuse the entry and exit lanes — Gates 3 and 5 are planned for exit only.</v>
+        <v>Park within your own allotted slot and inside the markings. No-parking zones and fire lanes are strictly enforced — vehicles are locked and fined Rs 200 a day for two-wheelers and Rs 500 for four-wheelers. No waste or storage in parking areas, and cycles belong in flat parking only.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Swimming pool usage rules</v>
+        <v>Security at the main gate</v>
       </c>
       <c r="B6" t="str">
-        <v>poster-pool.jpg</v>
+        <v>poster-gate-security.jpg</v>
       </c>
       <c r="C6" t="str">
-        <v>Proper swimwear is mandatory. Children must be supervised by an adult at all times. No food or glass items near the pool. The pool is for registered residents only — guests are not allowed.</v>
+        <v>Residents: affix the society sticker and register your vehicle for automatic access. Guests and non-registered vehicles must use Gate 1 for entry checks. Do not misuse the entry and exit lanes — Gates 3 and 5 are planned for exit only.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Gym guidelines</v>
+        <v>Swimming pool usage rules</v>
       </c>
       <c r="B7" t="str">
-        <v>poster-gym.jpg</v>
+        <v>poster-pool.jpg</v>
       </c>
       <c r="C7" t="str">
-        <v>Under-14s are not allowed in the gym. Do not drop weights or misuse equipment — place them gently and re-rack after use. Limit sessions to 30 minutes during peak hours so everyone gets a chance, and keep the shared audio at a moderate volume.</v>
+        <v>Proper swimwear is mandatory. Children must be supervised by an adult at all times. No food or glass items near the pool. The pool is for registered residents only — guests are not allowed.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Residents’ behaviour towards support staff</v>
+        <v>Gym guidelines</v>
       </c>
       <c r="B8" t="str">
-        <v>poster-staff-behaviour.jpg</v>
+        <v>poster-gym.jpg</v>
       </c>
       <c r="C8" t="str">
-        <v>Treat all support staff with dignity and courtesy — a smile and kind words go a long way. Do not be rude, dismissive or abusive towards support staff; mistreating them creates an unhealthy environment and is serious misconduct.</v>
+        <v>Under-14s are not allowed in the gym. Do not drop weights or misuse equipment — place them gently and re-rack after use. Limit sessions to 30 minutes during peak hours so everyone gets a chance, and keep the shared audio at a moderate volume.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Resident &amp; support staff interaction</v>
+        <v>Residents’ behaviour towards support staff</v>
       </c>
       <c r="B9" t="str">
-        <v>poster-staff-interaction.jpg</v>
+        <v>poster-staff-behaviour.jpg</v>
       </c>
       <c r="C9" t="str">
-        <v>Support staff are valued members of our society’s ecosystem and courteous interaction is expected at all times. They may not be engaged for private work inside flats beyond their defined scope. Verbal abuse, intimidation or disrespectful behaviour is strictly unacceptable — report any misconduct to the Maintenance Manager or Core Committee.</v>
+        <v>Treat all support staff with dignity and courtesy — a smile and kind words go a long way. Do not be rude, dismissive or abusive towards support staff; mistreating them creates an unhealthy environment and is serious misconduct.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
+        <v>Resident &amp; support staff interaction</v>
+      </c>
+      <c r="B10" t="str">
+        <v>poster-staff-interaction.jpg</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Support staff are valued members of our society’s ecosystem and courteous interaction is expected at all times. They may not be engaged for private work inside flats beyond their defined scope. Verbal abuse, intimidation or disrespectful behaviour is strictly unacceptable — report any misconduct to the Maintenance Manager or Core Committee.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v>Save water — use it judiciously</v>
       </c>
-      <c r="B10" t="str">
+      <c r="B11" t="str">
         <v>poster-savewater.png</v>
       </c>
-      <c r="C10" t="str">
+      <c r="C11" t="str">
         <v>Boond boond se banta hai kal ka savera. Close taps when not in use, use a bucket instead of a shower, run full loads in washing machines, report leaks promptly, and water plants in the morning or evening.</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C10"/>
+  <autoFilter ref="A1:C11"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
stop pointing at posters that are no longer there
The posters now come from the sheet alone, so the ten figures still baked
into the page were referencing image files that no longer exist. Clear the
grid out and follow the pattern the events carousel already uses: the
section and its menu entry stay hidden until the sheet has something to
put in them, so a sheet outage never leaves an empty shelf on the page.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -41,7 +41,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="13">'checklist'!A1:B9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14">'downloads'!A1:C6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15">'gallery'!A1:E9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16">'posters'!A1:C11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16">'posters'!A1:C1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17">'events'!A1:E1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18">'improvements'!A1:D19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19">'resolutions'!A1:F9</definedName>
@@ -2554,7 +2554,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C1"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -2572,120 +2572,10 @@
         <v>caption</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>The portal, in your pocket – in one tap</v>
-      </c>
-      <c r="B2" t="str">
-        <v>poster-portal-launch.png</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Our Resident Information Portal is now live at shwetashubham.in — everything about the society in your pocket. The guidelines in full with a search box, amenity timings, helpline numbers you can tap to call, the approved fees and penalty schedule, the committee directory, meeting minutes, notices and resolutions, these posters and the new resident checklist. No login, no app store, no charge. One tap adds it to your home screen, where it opens like an app and stays readable even with no signal. The phone in the picture shows exactly how the icon will look once you have added it.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Balcony safety &amp; cleanliness</v>
-      </c>
-      <c r="B3" t="str">
-        <v>poster-balcony.jpg</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Balcony safety &amp; cleanliness — keep your balcony clean and contained, and never throw water, dust, cigarette butts or waste from balconies</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Corridors must be kept clean &amp; clear</v>
-      </c>
-      <c r="B4" t="str">
-        <v>poster-corridors.jpg</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Corridors must be kept clean &amp; clear — no footwear, cycles, furniture or storage in the common corridors. Keep the passage tidy and unobstructed for everyone.</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Parking rules</v>
-      </c>
-      <c r="B5" t="str">
-        <v>poster-parking.jpg</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Park within your own allotted slot and inside the markings. No-parking zones and fire lanes are strictly enforced — vehicles are locked and fined Rs 200 a day for two-wheelers and Rs 500 for four-wheelers. No waste or storage in parking areas, and cycles belong in flat parking only.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Security at the main gate</v>
-      </c>
-      <c r="B6" t="str">
-        <v>poster-gate-security.jpg</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Residents: affix the society sticker and register your vehicle for automatic access. Guests and non-registered vehicles must use Gate 1 for entry checks. Do not misuse the entry and exit lanes — Gates 3 and 5 are planned for exit only.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Swimming pool usage rules</v>
-      </c>
-      <c r="B7" t="str">
-        <v>poster-pool.jpg</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Proper swimwear is mandatory. Children must be supervised by an adult at all times. No food or glass items near the pool. The pool is for registered residents only — guests are not allowed.</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Gym guidelines</v>
-      </c>
-      <c r="B8" t="str">
-        <v>poster-gym.jpg</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Under-14s are not allowed in the gym. Do not drop weights or misuse equipment — place them gently and re-rack after use. Limit sessions to 30 minutes during peak hours so everyone gets a chance, and keep the shared audio at a moderate volume.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Residents’ behaviour towards support staff</v>
-      </c>
-      <c r="B9" t="str">
-        <v>poster-staff-behaviour.jpg</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Treat all support staff with dignity and courtesy — a smile and kind words go a long way. Do not be rude, dismissive or abusive towards support staff; mistreating them creates an unhealthy environment and is serious misconduct.</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Resident &amp; support staff interaction</v>
-      </c>
-      <c r="B10" t="str">
-        <v>poster-staff-interaction.jpg</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Support staff are valued members of our society’s ecosystem and courteous interaction is expected at all times. They may not be engaged for private work inside flats beyond their defined scope. Verbal abuse, intimidation or disrespectful behaviour is strictly unacceptable — report any misconduct to the Maintenance Manager or Core Committee.</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Save water — use it judiciously</v>
-      </c>
-      <c r="B11" t="str">
-        <v>poster-savewater.png</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Boond boond se banta hai kal ka savera. Close taps when not in use, use a bucket instead of a shower, run full loads in washing machines, report leaks promptly, and water plants in the morning or evening.</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:C11"/>
+  <autoFilter ref="A1:C1"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
add the national cyber crime helpline to the numbers
Online fraud and UPI scams are the complaint residents are most likely to
face and least likely to know where to report, so 1930 now sits with the
other support numbers, tap-to-call like the rest.

The three helpline tests that pinned the built-in count at eleven now
count the cards in the page instead, so adding a number does not break
them again.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -30,7 +30,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2">'notices'!A1:D4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3">'festivals'!A1:B15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4">'quick_actions'!A1:D11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5">'helplines'!A1:E12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5">'helplines'!A1:E13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6">'timings'!A1:C11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7">'gates'!A1:C10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8">'guidelines'!A1:F139</definedName>
@@ -3754,7 +3754,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -3967,10 +3967,27 @@
         <v>Round-the-clock support and assistance for women.</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Support</v>
+      </c>
+      <c r="B13" t="str">
+        <v>🔒</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Cyber security</v>
+      </c>
+      <c r="D13" t="str">
+        <v>1930</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Online fraud, UPI scams and cyber crime — call as soon as it happens.</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E12"/>
+  <autoFilter ref="A1:E13"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
stop letting Google decide where the headings stop
Edits to the sheet were silently vanishing. Without headers=1 the gviz
export guesses how many opening rows are headings by looking at the
column types, and one clean number in a column of mixed text is enough
for it to guess wrong: adding 1930 to the helplines tab made it fold all
eleven rows above into a single heading row and return one record, so
the renderer rejected the lot and fell back to the page.

Pin the heading row to one and the same tab returns all twelve records.
Every tab is affected, not just helplines, and the failure is silent
either way.

The two test harnesses read the tab name by splitting on sheet=, which
breaks the moment another parameter follows, so both now match it
properly. The built-in card is renamed to match the sheet.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -3969,13 +3969,13 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Support</v>
+        <v>Emergency</v>
       </c>
       <c r="B13" t="str">
         <v>🔒</v>
       </c>
       <c r="C13" t="str">
-        <v>Cyber security</v>
+        <v>Cyber Fraud</v>
       </c>
       <c r="D13" t="str">
         <v>1930</v>

</xml_diff>

<commit_message>
Link the society memories archive from the resident portal
Add a responsive photograph card after Latest events and a Memories footer link. Both open the existing Google Site in a new tab, keeping the portal available. Reuse the settings hooks for an optional memories_url override, include it in the generated workbook and admin guide, and refresh the offline shell version.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -26,7 +26,7 @@
     <sheet name="records" sheetId="21" r:id="rId21"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'settings'!A1:B14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'settings'!A1:B15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2">'notices'!A1:D4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3">'festivals'!A1:B15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4">'quick_actions'!A1:D11</definedName>
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B85"/>
+  <dimension ref="A1:B86"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="78.83203125" customWidth="1"/>
@@ -554,445 +554,453 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>notices</v>
+        <v>settings: memories_url</v>
       </c>
       <c r="B20" t="str">
-        <v>The notice board. Newest at the top. colour = red / gold / green / grey</v>
+        <v>The SS Memories archive link used by the Memories card and footer. Leave this row out to keep the built-in archive address.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>festivals</v>
+        <v>notices</v>
       </c>
       <c r="B21" t="str">
-        <v>The festival chips under 'Celebrations we share'</v>
+        <v>The notice board. Newest at the top. colour = red / gold / green / grey</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>quick_actions</v>
+        <v>festivals</v>
       </c>
       <c r="B22" t="str">
-        <v>The eight shortcut tiles near the top of the page</v>
+        <v>The festival chips under 'Celebrations we share'</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>timings</v>
+        <v>quick_actions</v>
       </c>
       <c r="B23" t="str">
-        <v>The timings quick-reference table</v>
+        <v>The eight shortcut tiles near the top of the page</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>guidelines</v>
+        <v>timings</v>
       </c>
       <c r="B24" t="str">
-        <v>The full rulebook. See the note below.</v>
+        <v>The timings quick-reference table</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>staff_scope</v>
+        <v>guidelines</v>
       </c>
       <c r="B25" t="str">
-        <v>What the electrician, plumber, housekeeping, gardener and security cover</v>
+        <v>The full rulebook. See the note below.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>fees</v>
+        <v>staff_scope</v>
       </c>
       <c r="B26" t="str">
-        <v>type=card for the three summary boxes, type=penalty for the fines table</v>
+        <v>What the electrician, plumber, housekeeping, gardener and security cover</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>committee</v>
+        <v>fees</v>
       </c>
       <c r="B27" t="str">
-        <v>group = core / advisory / extended</v>
+        <v>type=card for the three summary boxes, type=penalty for the fines table</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>gates</v>
+        <v>committee</v>
       </c>
       <c r="B28" t="str">
-        <v>Which gate is open, when, and to whom. Repeat the gate name on each of its rows.</v>
+        <v>group = core / advisory / extended</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>escalation</v>
+        <v>gates</v>
       </c>
       <c r="B29" t="str">
-        <v>Who to contact, in order</v>
+        <v>Which gate is open, when, and to whom. Repeat the gate name on each of its rows.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>checklist</v>
+        <v>escalation</v>
       </c>
       <c r="B30" t="str">
-        <v>The new-resident checklist. Numbering is automatic.</v>
+        <v>Who to contact, in order</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>downloads</v>
+        <v>checklist</v>
       </c>
       <c r="B31" t="str">
-        <v>Forms and documents. Paste a Google Drive share link in url, or a file name kept beside the website.</v>
+        <v>The new-resident checklist. Numbering is automatic.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>gallery</v>
+        <v>downloads</v>
       </c>
       <c r="B32" t="str">
-        <v>Photos. Paste a Google Drive share link in file, or use an images folder file name.</v>
+        <v>Forms and documents. Paste a Google Drive share link in url, or a file name kept beside the website.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>posters</v>
+        <v>gallery</v>
       </c>
       <c r="B33" t="str">
-        <v>Tall 9:16 guideline posters. Use a Google Drive link, or the image file name.</v>
+        <v>Photos. Paste a Google Drive share link in file, or use an images folder file name.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>events</v>
+        <v>posters</v>
       </c>
       <c r="B34" t="str">
-        <v>Photographs from society events. See the note below.</v>
+        <v>Tall 9:16 guideline posters. Use a Google Drive link, or the image file name.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>improvements</v>
+        <v>events</v>
       </c>
       <c r="B35" t="str">
-        <v>Infrastructure and facilities created by SSMACS. title, category, year, details. No photo.</v>
+        <v>Photographs from society events. See the note below.</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>resolutions</v>
+        <v>improvements</v>
       </c>
       <c r="B36" t="str">
-        <v>Committee / GBM decisions. Newest first is not required — the site sorts by date.</v>
+        <v>Infrastructure and facilities created by SSMACS. title, category, year, details. No photo.</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>records</v>
+        <v>resolutions</v>
       </c>
       <c r="B37" t="str">
-        <v>Minutes of meetings, notices and circulars. See the note below.</v>
+        <v>Committee / GBM decisions. Newest first is not required — the site sorts by date.</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v/>
+        <v>records</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Minutes of meetings, notices and circulars. See the note below.</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>ABOUT THE EVENTS TAB</v>
+        <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>name</v>
-      </c>
-      <c r="B40" t="str">
-        <v>The event, e.g. Ganesh Chaturthi 2026. A row with no name is skipped.</v>
+        <v>ABOUT THE EVENTS TAB</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>date</v>
+        <v>name</v>
       </c>
       <c r="B41" t="str">
-        <v>Type it as 2026-09-14 (year-month-day). The newest event is shown first.</v>
+        <v>The event, e.g. Ganesh Chaturthi 2026. A row with no name is skipped.</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>details</v>
+        <v>date</v>
       </c>
       <c r="B42" t="str">
-        <v>A sentence or two about the day. Optional.</v>
+        <v>Type it as 2026-09-14 (year-month-day). The newest event is shown first.</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>photo</v>
+        <v>details</v>
       </c>
       <c r="B43" t="str">
-        <v>The Google Drive link to the picture. Leave blank if the row has a video.</v>
+        <v>A sentence or two about the day. Optional.</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>video</v>
+        <v>photo</v>
       </c>
       <c r="B44" t="str">
-        <v>The Google Drive link to a video, or a YouTube link. Optional.</v>
+        <v>The Google Drive link to the picture. Leave blank if the row has a video.</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v/>
+        <v>video</v>
+      </c>
+      <c r="B45" t="str">
+        <v>The Google Drive link to a video, or a YouTube link. Optional.</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>A row needs a name and either a photo or a video. A video slide shows a still</v>
+        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>from the film with a play button; tapping it plays the film full screen.</v>
+        <v>A row needs a name and either a photo or a video. A video slide shows a still</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v/>
+        <v>from the film with a play button; tapping it plays the film full screen.</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>IMPORTANT: each picture in Drive must be shared as</v>
+        <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v/>
-      </c>
-      <c r="B50" t="str">
-        <v>Share -&gt; General access -&gt; Anyone with the link -&gt; Viewer.</v>
+        <v>IMPORTANT: each picture in Drive must be shared as</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Without that the picture is private and residents see a placeholder.</v>
+        <v/>
+      </c>
+      <c r="B51" t="str">
+        <v>Share -&gt; General access -&gt; Anyone with the link -&gt; Viewer.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Paste the ordinary Drive share link. The website converts it itself.</v>
+        <v>Without that the picture is private and residents see a placeholder.</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>The section stays hidden until this tab has at least one complete row.</v>
+        <v>Paste the ordinary Drive share link. The website converts it itself.</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>The posters and gallery tabs take Drive links in the same way, same sharing rule.</v>
+        <v>The section stays hidden until this tab has at least one complete row.</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v/>
+        <v>The posters and gallery tabs take Drive links in the same way, same sharing rule.</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>ABOUT THE RESOLUTIONS TAB</v>
+        <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>date</v>
-      </c>
-      <c r="B57" t="str">
-        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
+        <v>ABOUT THE RESOLUTIONS TAB</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>status</v>
+        <v>date</v>
       </c>
       <c r="B58" t="str">
-        <v>Passed / Approved / Noted / Deferred / Pending / Rejected — this sets the colour.</v>
+        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>link</v>
+        <v>status</v>
       </c>
       <c r="B59" t="str">
-        <v>Optional. A link to the full resolution PDF. Leave blank if there isn't one.</v>
+        <v>Passed / Approved / Noted / Deferred / Pending / Rejected — this sets the colour.</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>The 'Latest' button shows the five most recent; 'All' shows everything.</v>
+        <v>link</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Optional. A link to the full resolution PDF. Leave blank if there isn't one.</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v/>
+        <v>The 'Latest' button shows the five most recent; 'All' shows everything.</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>ABOUT THE RECORDS TAB</v>
+        <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>type</v>
-      </c>
-      <c r="B63" t="str">
-        <v>mom = minutes of meeting, notice, or circular. This drives the filter buttons.</v>
+        <v>ABOUT THE RECORDS TAB</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>date</v>
+        <v>type</v>
       </c>
       <c r="B64" t="str">
-        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
+        <v>mom = minutes of meeting, notice, or circular. This drives the filter buttons.</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>link</v>
+        <v>date</v>
       </c>
       <c r="B65" t="str">
-        <v>The PDF file name, e.g. gbm-april-2025.pdf, uploaded next to the website.</v>
+        <v>Type it as 2025-04-26 (year-month-day). Format the column as Plain text.</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Leave link blank and the row points at the contact section instead.</v>
+        <v>link</v>
+      </c>
+      <c r="B66" t="str">
+        <v>The PDF file name, e.g. gbm-april-2025.pdf, uploaded next to the website.</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v/>
+        <v>Leave link blank and the row points at the contact section instead.</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>ABOUT THE GUIDELINES TAB</v>
+        <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Each rule section is several rows sharing the same 'section' number.</v>
+        <v>ABOUT THE GUIDELINES TAB</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Fill in title, keywords and anchor on the FIRST row of a section only.</v>
+        <v>Each rule section is several rows sharing the same 'section' number.</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>The 'kind' column decides how the row looks:</v>
+        <v>Fill in title, keywords and anchor on the FIRST row of a section only.</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>li</v>
-      </c>
-      <c r="B72" t="str">
-        <v>a normal bullet point</v>
+        <v>The 'kind' column decides how the row looks:</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>sub</v>
+        <v>li</v>
       </c>
       <c r="B73" t="str">
-        <v>a bold sub-heading, e.g. 'Gym' inside the Sports section</v>
+        <v>a normal bullet point</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>note</v>
+        <v>sub</v>
       </c>
       <c r="B74" t="str">
-        <v>a grey highlighted box</v>
+        <v>a bold sub-heading, e.g. 'Gym' inside the Sports section</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>note-red</v>
+        <v>note</v>
       </c>
       <c r="B75" t="str">
-        <v>a red warning box</v>
+        <v>a grey highlighted box</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>note-green</v>
+        <v>note-red</v>
       </c>
       <c r="B76" t="str">
-        <v>a green box</v>
+        <v>a red warning box</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>p</v>
+        <v>note-green</v>
       </c>
       <c r="B77" t="str">
-        <v>an ordinary paragraph</v>
+        <v>a green box</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v/>
+        <v>p</v>
+      </c>
+      <c r="B78" t="str">
+        <v>an ordinary paragraph</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>'keywords' are extra words the website search should match for that section.</v>
+        <v/>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v/>
+        <v>'keywords' are extra words the website search should match for that section.</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>IF SOMETHING GOES WRONG</v>
+        <v/>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>The website falls back to its built-in copy if this sheet cannot be read,</v>
+        <v>IF SOMETHING GOES WRONG</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>so a mistake here can never take the site down. Undo the change and refresh.</v>
+        <v>The website falls back to its built-in copy if this sheet cannot be read,</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v/>
+        <v>so a mistake here can never take the site down. Undo the change and refresh.</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
         <v>Remember: Share -&gt; Anyone with the link -&gt; Viewer, or the website cannot read this.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B85"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B86"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2902,7 +2910,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="70.83203125" customWidth="1"/>
@@ -3014,16 +3022,24 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
+        <v>memories_url</v>
+      </c>
+      <c r="B14" t="str">
+        <v>https://sites.google.com/view/ssmemories/home</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
         <v>map_embed</v>
       </c>
-      <c r="B14" t="str">
+      <c r="B15" t="str">
         <v>https://maps.google.com/maps?q=Shweta+Shubham,+Kompally,+Hyderabad&amp;z=16&amp;hl=en&amp;output=embed</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B14"/>
+  <autoFilter ref="A1:B15"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add owner and tenant sign-off PDF
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -2341,10 +2341,10 @@
         <v>Owner &amp; tenant sign-off proforma</v>
       </c>
       <c r="B3" t="str">
-        <v>Collect from the society office</v>
+        <v>Download, print, sign and submit to the society office</v>
       </c>
       <c r="C3" t="str">
-        <v>#contact</v>
+        <v>forms/owner-tenant-signoff-proforma.pdf</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Add vehicle registration PDF form
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -2352,10 +2352,10 @@
         <v>Vehicle registration form</v>
       </c>
       <c r="B4" t="str">
-        <v>Required for Gate 2 boom barrier access</v>
+        <v>Download and submit with the RC copy for Gate 2 boom barrier access</v>
       </c>
       <c r="C4" t="str">
-        <v>#contact</v>
+        <v>forms/vehicle-registration-form.pdf</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Add NOC request PDF form
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -2363,10 +2363,10 @@
         <v>NOC request — resale / move-out</v>
       </c>
       <c r="B5" t="str">
-        <v>Issued by the society office</v>
+        <v>Download, complete and submit for society clearance</v>
       </c>
       <c r="C5" t="str">
-        <v>#contact</v>
+        <v>forms/noc-request-resale-move-out.pdf</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Add pet vaccination PDF form
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -2374,10 +2374,10 @@
         <v>Pet vaccination certificate submission</v>
       </c>
       <c r="B6" t="str">
-        <v>To be submitted regularly to the society office</v>
+        <v>Download and submit with the pet's current vaccination certificate</v>
       </c>
       <c r="C6" t="str">
-        <v>#contact</v>
+        <v>forms/pet-vaccination-certificate-submission.pdf</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add tenant move-in to NOC form
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -2360,13 +2360,13 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>NOC request — resale / move-out</v>
+        <v>NOC request — resale / move-in / move-out</v>
       </c>
       <c r="B5" t="str">
-        <v>Download, complete and submit for society clearance</v>
+        <v>Includes required tenant photo, Aadhaar and move-in documents</v>
       </c>
       <c r="C5" t="str">
-        <v>forms/noc-request-resale-move-out.pdf</v>
+        <v>forms/noc-request-resale-move-in-move-out.pdf</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Add tenant no-pet move-in policy
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Shweta-Shubham-Content.xlsx
+++ b/Shweta-Shubham-Content.xlsx
@@ -33,7 +33,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5">'helplines'!A1:E13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6">'timings'!A1:C11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7">'gates'!A1:C10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8">'guidelines'!A1:F139</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8">'guidelines'!A1:F140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9">'staff_scope'!A1:D37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10">'fees'!A1:E17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11">'committee'!A1:F21</definedName>
@@ -2267,10 +2267,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Pet registration</v>
+        <v>Pet policy</v>
       </c>
       <c r="B6" t="str">
-        <v>Submit a copy of the valid vaccination certificate to the society office, if applicable.</v>
+        <v>Tenants cannot keep pets. Owners with pets must submit a valid vaccination certificate.</v>
       </c>
     </row>
     <row r="7">
@@ -4278,7 +4278,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F139"/>
+  <dimension ref="A1:F140"/>
   <cols>
     <col min="1" max="1" width="9.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -5527,7 +5527,7 @@
         <v>li</v>
       </c>
       <c r="F108" t="str">
-        <v>Pets must be on a leash and accompanied by the owner at all times; use of a muzzle is mandatory.</v>
+        <v>**Only flat owners may keep pets. Tenants are not permitted to keep pets.**</v>
       </c>
     </row>
     <row r="109">
@@ -5538,7 +5538,7 @@
         <v>li</v>
       </c>
       <c r="F109" t="str">
-        <v>Owners must ensure pets do not cause disturbance, such as excessive barking.</v>
+        <v>Pets must be on a leash and accompanied by the owner at all times; use of a muzzle is mandatory.</v>
       </c>
     </row>
     <row r="110">
@@ -5549,7 +5549,7 @@
         <v>li</v>
       </c>
       <c r="F110" t="str">
-        <v>A copy of a valid vaccination certificate must be regularly submitted to the society office.</v>
+        <v>Owners must ensure pets do not cause disturbance, such as excessive barking.</v>
       </c>
     </row>
     <row r="111">
@@ -5560,7 +5560,7 @@
         <v>li</v>
       </c>
       <c r="F111" t="str">
-        <v>Pet owners must clean up pet waste in common areas and are responsible for any damage caused by their pets.</v>
+        <v>A copy of a valid vaccination certificate must be regularly submitted to the society office.</v>
       </c>
     </row>
     <row r="112">
@@ -5571,7 +5571,7 @@
         <v>li</v>
       </c>
       <c r="F112" t="str">
-        <v>Pets may not roam freely in corridors or lifts, and are not permitted on rooftops or in the pool area.</v>
+        <v>Pet owners must clean up pet waste in common areas and are responsible for any damage caused by their pets.</v>
       </c>
     </row>
     <row r="113">
@@ -5579,38 +5579,38 @@
         <v>7</v>
       </c>
       <c r="E113" t="str">
-        <v>note-red</v>
+        <v>li</v>
       </c>
       <c r="F113" t="str">
-        <v>All pet policy violations attract a fine of ₹1,000.</v>
+        <v>Pets may not roam freely in corridors or lifts, and are not permitted on rooftops or in the pool area.</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>8</v>
-      </c>
-      <c r="B114" t="str">
-        <v>Waste Management &amp; Cleanliness</v>
-      </c>
-      <c r="C114" t="str">
-        <v>waste management cleanliness dustbin spitting diapers sanitary napkins garbage</v>
+        <v>7</v>
       </c>
       <c r="E114" t="str">
-        <v>li</v>
+        <v>note-red</v>
       </c>
       <c r="F114" t="str">
-        <v>Closed-lid dustbins must be used by residents.</v>
+        <v>All pet policy violations attract a fine of ₹1,000.</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
         <v>8</v>
       </c>
+      <c r="B115" t="str">
+        <v>Waste Management &amp; Cleanliness</v>
+      </c>
+      <c r="C115" t="str">
+        <v>waste management cleanliness dustbin spitting diapers sanitary napkins garbage</v>
+      </c>
       <c r="E115" t="str">
         <v>li</v>
       </c>
       <c r="F115" t="str">
-        <v>Dumping waste in common areas or parking areas is strictly prohibited.</v>
+        <v>Closed-lid dustbins must be used by residents.</v>
       </c>
     </row>
     <row r="116">
@@ -5621,7 +5621,7 @@
         <v>li</v>
       </c>
       <c r="F116" t="str">
-        <v>Waste removal charges, along with applicable fines, will be charged to the respective flat.</v>
+        <v>Dumping waste in common areas or parking areas is strictly prohibited.</v>
       </c>
     </row>
     <row r="117">
@@ -5632,7 +5632,7 @@
         <v>li</v>
       </c>
       <c r="F117" t="str">
-        <v>Spitting is prohibited — a fine of ₹1,000 will be imposed.</v>
+        <v>Waste removal charges, along with applicable fines, will be charged to the respective flat.</v>
       </c>
     </row>
     <row r="118">
@@ -5643,7 +5643,7 @@
         <v>li</v>
       </c>
       <c r="F118" t="str">
-        <v>Disposing of diapers or sanitary napkins via the flush is prohibited.</v>
+        <v>Spitting is prohibited — a fine of ₹1,000 will be imposed.</v>
       </c>
     </row>
     <row r="119">
@@ -5651,38 +5651,38 @@
         <v>8</v>
       </c>
       <c r="E119" t="str">
-        <v>note-red</v>
+        <v>li</v>
       </c>
       <c r="F119" t="str">
-        <v>All violators shall be fined ₹1,000.</v>
+        <v>Disposing of diapers or sanitary napkins via the flush is prohibited.</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>9</v>
-      </c>
-      <c r="B120" t="str">
-        <v>Children &amp; Minor Safety</v>
-      </c>
-      <c r="C120" t="str">
-        <v>children minor safety lift pool play area tot lot supervision parent guardian</v>
+        <v>8</v>
       </c>
       <c r="E120" t="str">
-        <v>li</v>
+        <v>note-red</v>
       </c>
       <c r="F120" t="str">
-        <v>**Lifts** — children below 8 years must be accompanied by a parent or guardian.</v>
+        <v>All violators shall be fined ₹1,000.</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
         <v>9</v>
       </c>
+      <c r="B121" t="str">
+        <v>Children &amp; Minor Safety</v>
+      </c>
+      <c r="C121" t="str">
+        <v>children minor safety lift pool play area tot lot supervision parent guardian</v>
+      </c>
       <c r="E121" t="str">
         <v>li</v>
       </c>
       <c r="F121" t="str">
-        <v>**Swimming pool** — children below 12 must be with a parent or guardian; non-swimmers must be accompanied by a competent adult.</v>
+        <v>**Lifts** — children below 8 years must be accompanied by a parent or guardian.</v>
       </c>
     </row>
     <row r="122">
@@ -5693,7 +5693,7 @@
         <v>li</v>
       </c>
       <c r="F122" t="str">
-        <v>**Play area** — ensure fair usage and equal opportunity for others; adherence to designated timings is mandatory.</v>
+        <v>**Swimming pool** — children below 12 must be with a parent or guardian; non-swimmers must be accompanied by a competent adult.</v>
       </c>
     </row>
     <row r="123">
@@ -5704,35 +5704,35 @@
         <v>li</v>
       </c>
       <c r="F123" t="str">
-        <v>**Tot-lots and parks** — cycling, skating and playing with hard balls are strictly prohibited.</v>
+        <v>**Play area** — ensure fair usage and equal opportunity for others; adherence to designated timings is mandatory.</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>10</v>
-      </c>
-      <c r="B124" t="str">
-        <v>Noise &amp; Quiet Hours</v>
-      </c>
-      <c r="C124" t="str">
-        <v>noise quiet hours music decorum 10 pm carpentry</v>
+        <v>9</v>
       </c>
       <c r="E124" t="str">
         <v>li</v>
       </c>
       <c r="F124" t="str">
-        <v>Loud noise, music or gatherings should be avoided after **10:00 PM**.</v>
+        <v>**Tot-lots and parks** — cycling, skating and playing with hard balls are strictly prohibited.</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
         <v>10</v>
       </c>
+      <c r="B125" t="str">
+        <v>Noise &amp; Quiet Hours</v>
+      </c>
+      <c r="C125" t="str">
+        <v>noise quiet hours music decorum 10 pm carpentry</v>
+      </c>
       <c r="E125" t="str">
         <v>li</v>
       </c>
       <c r="F125" t="str">
-        <v>Swimming pool — maintain silence and decorum; no music or disturbance.</v>
+        <v>Loud noise, music or gatherings should be avoided after **10:00 PM**.</v>
       </c>
     </row>
     <row r="126">
@@ -5743,7 +5743,7 @@
         <v>li</v>
       </c>
       <c r="F126" t="str">
-        <v>Indoor games — do not disturb other users or create excessive noise.</v>
+        <v>Swimming pool — maintain silence and decorum; no music or disturbance.</v>
       </c>
     </row>
     <row r="127">
@@ -5754,7 +5754,7 @@
         <v>li</v>
       </c>
       <c r="F127" t="str">
-        <v>Gym — keep volume on the shared music system moderate.</v>
+        <v>Indoor games — do not disturb other users or create excessive noise.</v>
       </c>
     </row>
     <row r="128">
@@ -5765,7 +5765,7 @@
         <v>li</v>
       </c>
       <c r="F128" t="str">
-        <v>Corridors and common areas — maintain cleanliness and proper decorum at all times.</v>
+        <v>Gym — keep volume on the shared music system moderate.</v>
       </c>
     </row>
     <row r="129">
@@ -5776,35 +5776,35 @@
         <v>li</v>
       </c>
       <c r="F129" t="str">
-        <v>Carpentry and in-house works only between 9:00 AM and 7:00 PM.</v>
+        <v>Corridors and common areas — maintain cleanliness and proper decorum at all times.</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>7.4</v>
-      </c>
-      <c r="B130" t="str">
-        <v>Move-In / Move-Out Process</v>
-      </c>
-      <c r="C130" t="str">
-        <v>move in move out shifting proforma noc gate pass luggage vehicle east driveway 1000</v>
+        <v>10</v>
       </c>
       <c r="E130" t="str">
         <v>li</v>
       </c>
       <c r="F130" t="str">
-        <v>Give prior information to the Maintenance Manager before moving in or out.</v>
+        <v>Carpentry and in-house works only between 9:00 AM and 7:00 PM.</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
         <v>7.4</v>
       </c>
+      <c r="B131" t="str">
+        <v>Move-In / Move-Out Process</v>
+      </c>
+      <c r="C131" t="str">
+        <v>move in move out shifting proforma noc gate pass luggage vehicle east driveway 1000</v>
+      </c>
       <c r="E131" t="str">
         <v>li</v>
       </c>
       <c r="F131" t="str">
-        <v>Produce the signed proforma by both owner and tenant before moving in.</v>
+        <v>Give prior information to the Maintenance Manager before moving in or out.</v>
       </c>
     </row>
     <row r="132">
@@ -5815,7 +5815,7 @@
         <v>li</v>
       </c>
       <c r="F132" t="str">
-        <v>Shifting is permitted only between **7:00 AM and 6:00 PM**.</v>
+        <v>Produce the signed proforma by both owner and tenant before moving in.</v>
       </c>
     </row>
     <row r="133">
@@ -5826,7 +5826,7 @@
         <v>li</v>
       </c>
       <c r="F133" t="str">
-        <v>**₹1,000** is charged each for move-in and move-out (applicable to tenants).</v>
+        <v>Shifting is permitted only between **7:00 AM and 6:00 PM**.</v>
       </c>
     </row>
     <row r="134">
@@ -5837,7 +5837,7 @@
         <v>li</v>
       </c>
       <c r="F134" t="str">
-        <v>Move-out requires an NOC from the Maintenance Manager with owner confirmation for gate pass issuance.</v>
+        <v>**₹1,000** is charged each for move-in and move-out (applicable to tenants).</v>
       </c>
     </row>
     <row r="135">
@@ -5848,35 +5848,35 @@
         <v>li</v>
       </c>
       <c r="F135" t="str">
-        <v>The luggage vehicle must be parked so it does not inconvenience residents — only in designated areas on the East side driveway.</v>
+        <v>Move-out requires an NOC from the Maintenance Manager with owner confirmation for gate pass issuance.</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>1.4</v>
-      </c>
-      <c r="B136" t="str">
-        <v>Suggestions &amp; Support</v>
-      </c>
-      <c r="C136" t="str">
-        <v>suggestion box support complaint office weekend committee</v>
+        <v>7.4</v>
       </c>
       <c r="E136" t="str">
         <v>li</v>
       </c>
       <c r="F136" t="str">
-        <v>A suggestion box is available at the reception. Residents are encouraged to submit suggestions or complaints.</v>
+        <v>The luggage vehicle must be parked so it does not inconvenience residents — only in designated areas on the East side driveway.</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
         <v>1.4</v>
       </c>
+      <c r="B137" t="str">
+        <v>Suggestions &amp; Support</v>
+      </c>
+      <c r="C137" t="str">
+        <v>suggestion box support complaint office weekend committee</v>
+      </c>
       <c r="E137" t="str">
         <v>li</v>
       </c>
       <c r="F137" t="str">
-        <v>Contact the society office for maintenance support during working hours.</v>
+        <v>A suggestion box is available at the reception. Residents are encouraged to submit suggestions or complaints.</v>
       </c>
     </row>
     <row r="138">
@@ -5887,7 +5887,7 @@
         <v>li</v>
       </c>
       <c r="F138" t="str">
-        <v>In emergencies, contact any Committee Member.</v>
+        <v>Contact the society office for maintenance support during working hours.</v>
       </c>
     </row>
     <row r="139">
@@ -5898,13 +5898,24 @@
         <v>li</v>
       </c>
       <c r="F139" t="str">
+        <v>In emergencies, contact any Committee Member.</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>1.4</v>
+      </c>
+      <c r="E140" t="str">
+        <v>li</v>
+      </c>
+      <c r="F140" t="str">
         <v>Committee Members may be available at the office on weekends.</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F139"/>
+  <autoFilter ref="A1:F140"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F139"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F140"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>